<commit_message>
Updated and checked manure management data and added 'anaerobic digestion' and 'composting' as MMSs
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="206">
   <si>
     <t>f_crop</t>
   </si>
@@ -502,9 +502,6 @@
     <t>poultry</t>
   </si>
   <si>
-    <t>broiler</t>
-  </si>
-  <si>
     <t>liquid</t>
   </si>
   <si>
@@ -580,9 +577,6 @@
     <t>mineral N fertiliser</t>
   </si>
   <si>
-    <t>NH3 from manure on pasture!!</t>
-  </si>
-  <si>
     <t>applied manure</t>
   </si>
   <si>
@@ -653,6 +647,21 @@
   </si>
   <si>
     <t>Avg. from statistics 2018/2019 &amp; 2021/2022</t>
+  </si>
+  <si>
+    <t>anaerobic digestion</t>
+  </si>
+  <si>
+    <t>composting</t>
+  </si>
+  <si>
+    <t>sheep</t>
+  </si>
+  <si>
+    <t>laying chicks</t>
+  </si>
+  <si>
+    <t>broilers</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1061,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S300"/>
+  <dimension ref="A1:S317"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
@@ -1074,10 +1083,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>90</v>
@@ -1086,7 +1095,7 @@
         <v>8</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>136</v>
@@ -1178,7 +1187,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1201,7 +1210,7 @@
         <v>113</v>
       </c>
       <c r="L8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M8">
         <v>0</v>
@@ -1210,18 +1219,18 @@
         <v>127</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F9" t="s">
         <v>125</v>
       </c>
       <c r="L9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M9">
         <v>59</v>
@@ -1238,13 +1247,13 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F10" t="s">
         <v>126</v>
       </c>
       <c r="L10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M10">
         <v>7</v>
@@ -1258,13 +1267,13 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F11" t="s">
         <v>124</v>
       </c>
       <c r="L11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M11">
         <v>34</v>
@@ -2978,7 +2987,7 @@
       </c>
       <c r="N124" s="7"/>
       <c r="O124" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.25">
@@ -4885,7 +4894,7 @@
     </row>
     <row r="239" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B239" s="2"/>
       <c r="C239" s="2"/>
@@ -4908,7 +4917,7 @@
         <v>131</v>
       </c>
       <c r="L240" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M240" s="14">
         <v>0</v>
@@ -4917,12 +4926,12 @@
         <v>132</v>
       </c>
       <c r="O240" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="241" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B241" s="1"/>
       <c r="K241" s="6"/>
@@ -4939,7 +4948,7 @@
         <v>131</v>
       </c>
       <c r="L242" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M242" s="12">
         <f>8/1000*(14/(1*14+3*2))*100</f>
@@ -4963,7 +4972,7 @@
         <v>131</v>
       </c>
       <c r="L243" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M243" s="12">
         <f>15/1000*(14/(1*14+3*2))*100</f>
@@ -4984,7 +4993,7 @@
         <v>131</v>
       </c>
       <c r="L244" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M244" s="12">
         <f>50/1000*(14/(1*14+3*2))*100</f>
@@ -4999,11 +5008,11 @@
     </row>
     <row r="245" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B245" s="1"/>
       <c r="C245" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="246" spans="1:16" x14ac:dyDescent="0.25">
@@ -5017,13 +5026,13 @@
         <v>142</v>
       </c>
       <c r="J246" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K246" t="s">
         <v>131</v>
       </c>
       <c r="L246" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M246">
         <v>33</v>
@@ -5032,7 +5041,7 @@
         <v>132</v>
       </c>
       <c r="P246" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="247" spans="1:16" x14ac:dyDescent="0.25">
@@ -5046,13 +5055,13 @@
         <v>142</v>
       </c>
       <c r="J247" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K247" t="s">
         <v>131</v>
       </c>
       <c r="L247" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M247">
         <v>38</v>
@@ -5061,7 +5070,7 @@
         <v>132</v>
       </c>
       <c r="P247" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="248" spans="1:16" x14ac:dyDescent="0.25">
@@ -5075,13 +5084,13 @@
         <v>142</v>
       </c>
       <c r="J248" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K248" t="s">
         <v>131</v>
       </c>
       <c r="L248" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M248">
         <v>41</v>
@@ -5090,7 +5099,7 @@
         <v>132</v>
       </c>
       <c r="P248" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="249" spans="1:16" x14ac:dyDescent="0.25">
@@ -5098,28 +5107,28 @@
         <v>140</v>
       </c>
       <c r="H249" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I249" t="s">
         <v>142</v>
       </c>
       <c r="J249" t="s">
-        <v>153</v>
+        <v>201</v>
       </c>
       <c r="K249" t="s">
         <v>131</v>
       </c>
       <c r="L249" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M249">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N249" t="s">
         <v>132</v>
       </c>
       <c r="P249" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="250" spans="1:16" x14ac:dyDescent="0.25">
@@ -5133,22 +5142,22 @@
         <v>142</v>
       </c>
       <c r="J250" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="K250" t="s">
         <v>131</v>
       </c>
       <c r="L250" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M250">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="N250" t="s">
         <v>132</v>
       </c>
       <c r="P250" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="251" spans="1:16" x14ac:dyDescent="0.25">
@@ -5162,74 +5171,80 @@
         <v>142</v>
       </c>
       <c r="J251" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="K251" t="s">
         <v>131</v>
       </c>
       <c r="L251" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M251">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="N251" t="s">
         <v>132</v>
       </c>
       <c r="P251" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="252" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G252" t="s">
         <v>140</v>
       </c>
+      <c r="H252" t="s">
+        <v>143</v>
+      </c>
       <c r="I252" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J252" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K252" t="s">
         <v>131</v>
       </c>
       <c r="L252" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M252">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="N252" t="s">
         <v>132</v>
       </c>
       <c r="P252" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="253" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G253" t="s">
         <v>140</v>
       </c>
+      <c r="H253" t="s">
+        <v>143</v>
+      </c>
       <c r="I253" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J253" t="s">
-        <v>154</v>
+        <v>201</v>
       </c>
       <c r="K253" t="s">
         <v>131</v>
       </c>
       <c r="L253" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M253">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="N253" t="s">
         <v>132</v>
       </c>
       <c r="P253" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="254" spans="1:16" x14ac:dyDescent="0.25">
@@ -5240,22 +5255,22 @@
         <v>144</v>
       </c>
       <c r="J254" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K254" t="s">
         <v>131</v>
       </c>
       <c r="L254" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M254">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="N254" t="s">
         <v>132</v>
       </c>
       <c r="P254" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="255" spans="1:16" x14ac:dyDescent="0.25">
@@ -5263,7 +5278,7 @@
         <v>140</v>
       </c>
       <c r="I255" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J255" t="s">
         <v>153</v>
@@ -5272,16 +5287,16 @@
         <v>131</v>
       </c>
       <c r="L255" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M255">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="N255" t="s">
         <v>132</v>
       </c>
       <c r="P255" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="256" spans="1:16" x14ac:dyDescent="0.25">
@@ -5289,7 +5304,7 @@
         <v>140</v>
       </c>
       <c r="I256" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J256" t="s">
         <v>154</v>
@@ -5298,16 +5313,16 @@
         <v>131</v>
       </c>
       <c r="L256" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M256">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="N256" t="s">
         <v>132</v>
       </c>
       <c r="P256" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="257" spans="7:16" x14ac:dyDescent="0.25">
@@ -5315,65 +5330,68 @@
         <v>140</v>
       </c>
       <c r="I257" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J257" t="s">
-        <v>155</v>
+        <v>201</v>
       </c>
       <c r="K257" t="s">
         <v>131</v>
       </c>
       <c r="L257" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M257">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="N257" t="s">
         <v>132</v>
       </c>
       <c r="P257" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="258" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G258" t="s">
         <v>140</v>
       </c>
+      <c r="I258" t="s">
+        <v>145</v>
+      </c>
       <c r="J258" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K258" t="s">
         <v>131</v>
       </c>
       <c r="L258" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M258">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N258" t="s">
         <v>132</v>
       </c>
-      <c r="O258" t="s">
-        <v>156</v>
-      </c>
       <c r="P258" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="259" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G259" t="s">
         <v>140</v>
       </c>
+      <c r="I259" t="s">
+        <v>145</v>
+      </c>
       <c r="J259" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K259" t="s">
         <v>131</v>
       </c>
       <c r="L259" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M259">
         <v>39</v>
@@ -5381,293 +5399,284 @@
       <c r="N259" t="s">
         <v>132</v>
       </c>
-      <c r="O259" t="s">
-        <v>156</v>
-      </c>
       <c r="P259" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="260" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G260" t="s">
         <v>140</v>
       </c>
+      <c r="I260" t="s">
+        <v>145</v>
+      </c>
       <c r="J260" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K260" t="s">
         <v>131</v>
       </c>
       <c r="L260" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M260">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N260" t="s">
         <v>132</v>
       </c>
-      <c r="O260" t="s">
-        <v>156</v>
-      </c>
       <c r="P260" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="261" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G261" t="s">
         <v>140</v>
       </c>
+      <c r="I261" t="s">
+        <v>145</v>
+      </c>
       <c r="J261" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="K261" t="s">
         <v>131</v>
       </c>
       <c r="L261" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M261">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="N261" t="s">
         <v>132</v>
       </c>
       <c r="P261" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
     </row>
     <row r="262" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G262" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="J262" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="K262" t="s">
         <v>131</v>
       </c>
       <c r="L262" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M262">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="N262" t="s">
         <v>132</v>
       </c>
+      <c r="O262" t="s">
+        <v>155</v>
+      </c>
       <c r="P262" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="263" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G263" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="J263" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="K263" t="s">
         <v>131</v>
       </c>
       <c r="L263" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M263">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N263" t="s">
         <v>132</v>
       </c>
+      <c r="O263" t="s">
+        <v>155</v>
+      </c>
       <c r="P263" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="264" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G264" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="J264" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="K264" t="s">
         <v>131</v>
       </c>
       <c r="L264" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M264">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N264" t="s">
         <v>132</v>
       </c>
+      <c r="O264" t="s">
+        <v>155</v>
+      </c>
       <c r="P264" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
     </row>
     <row r="265" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G265" t="s">
-        <v>146</v>
-      </c>
-      <c r="I265" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="J265" t="s">
-        <v>153</v>
+        <v>201</v>
       </c>
       <c r="K265" t="s">
         <v>131</v>
       </c>
       <c r="L265" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M265">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N265" t="s">
         <v>132</v>
       </c>
+      <c r="O265" t="s">
+        <v>155</v>
+      </c>
       <c r="P265" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="266" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G266" t="s">
-        <v>146</v>
-      </c>
-      <c r="I266" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="J266" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="K266" t="s">
         <v>131</v>
       </c>
       <c r="L266" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M266">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="N266" t="s">
         <v>132</v>
       </c>
       <c r="P266" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
     </row>
     <row r="267" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G267" t="s">
-        <v>146</v>
-      </c>
-      <c r="I267" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="J267" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="K267" t="s">
         <v>131</v>
       </c>
       <c r="L267" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M267">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="N267" t="s">
         <v>132</v>
       </c>
       <c r="P267" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="268" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G268" t="s">
-        <v>146</v>
-      </c>
-      <c r="I268" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="J268" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K268" t="s">
         <v>131</v>
       </c>
       <c r="L268" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M268">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="N268" t="s">
         <v>132</v>
       </c>
       <c r="P268" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="269" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G269" t="s">
-        <v>146</v>
-      </c>
-      <c r="I269" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="J269" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="K269" t="s">
         <v>131</v>
       </c>
       <c r="L269" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M269">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="N269" t="s">
         <v>132</v>
       </c>
       <c r="P269" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="270" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G270" t="s">
-        <v>146</v>
-      </c>
-      <c r="I270" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="J270" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="K270" t="s">
         <v>131</v>
       </c>
       <c r="L270" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M270">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="N270" t="s">
         <v>132</v>
       </c>
       <c r="P270" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
     </row>
     <row r="271" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G271" t="s">
-        <v>146</v>
-      </c>
-      <c r="I271" t="s">
-        <v>149</v>
+        <v>203</v>
       </c>
       <c r="J271" t="s">
         <v>153</v>
@@ -5676,76 +5685,73 @@
         <v>131</v>
       </c>
       <c r="L271" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M271">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="N271" t="s">
         <v>132</v>
       </c>
       <c r="P271" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="272" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G272" t="s">
-        <v>146</v>
-      </c>
-      <c r="I272" t="s">
-        <v>149</v>
+        <v>203</v>
       </c>
       <c r="J272" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="K272" t="s">
         <v>131</v>
       </c>
       <c r="L272" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M272">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="N272" t="s">
         <v>132</v>
       </c>
       <c r="P272" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="273" spans="1:16" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="273" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G273" t="s">
         <v>146</v>
       </c>
       <c r="I273" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J273" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K273" t="s">
         <v>131</v>
       </c>
       <c r="L273" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M273">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="N273" t="s">
         <v>132</v>
       </c>
       <c r="P273" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="274" spans="1:16" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="274" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G274" t="s">
         <v>146</v>
       </c>
       <c r="I274" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="J274" t="s">
         <v>153</v>
@@ -5754,28 +5760,24 @@
         <v>131</v>
       </c>
       <c r="L274" t="s">
-        <v>162</v>
-      </c>
-      <c r="M274" s="13">
-        <f>M265</f>
-        <v>30</v>
+        <v>161</v>
+      </c>
+      <c r="M274">
+        <v>35</v>
       </c>
       <c r="N274" t="s">
         <v>132</v>
       </c>
-      <c r="O274" t="s">
-        <v>158</v>
-      </c>
       <c r="P274" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="275" spans="1:16" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="275" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G275" t="s">
         <v>146</v>
       </c>
       <c r="I275" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="J275" t="s">
         <v>154</v>
@@ -5784,67 +5786,63 @@
         <v>131</v>
       </c>
       <c r="L275" t="s">
-        <v>162</v>
-      </c>
-      <c r="M275" s="13">
-        <f t="shared" ref="M275:M276" si="4">M266</f>
-        <v>35</v>
+        <v>161</v>
+      </c>
+      <c r="M275">
+        <v>48</v>
       </c>
       <c r="N275" t="s">
         <v>132</v>
       </c>
-      <c r="O275" t="s">
-        <v>158</v>
-      </c>
       <c r="P275" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="276" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G276" t="s">
         <v>146</v>
       </c>
       <c r="I276" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="J276" t="s">
-        <v>155</v>
+        <v>201</v>
       </c>
       <c r="K276" t="s">
         <v>131</v>
       </c>
       <c r="L276" t="s">
-        <v>162</v>
-      </c>
-      <c r="M276" s="13">
-        <f t="shared" si="4"/>
-        <v>48</v>
+        <v>161</v>
+      </c>
+      <c r="M276">
+        <v>30</v>
       </c>
       <c r="N276" t="s">
         <v>132</v>
       </c>
-      <c r="O276" t="s">
-        <v>158</v>
-      </c>
       <c r="P276" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="277" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G277" t="s">
         <v>146</v>
       </c>
+      <c r="I277" t="s">
+        <v>150</v>
+      </c>
       <c r="J277" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K277" t="s">
         <v>131</v>
       </c>
       <c r="L277" t="s">
-        <v>162</v>
-      </c>
-      <c r="M277">
-        <v>29</v>
+        <v>161</v>
+      </c>
+      <c r="M277" s="13">
+        <f>M273</f>
+        <v>30</v>
       </c>
       <c r="N277" t="s">
         <v>132</v>
@@ -5852,24 +5850,25 @@
       <c r="O277" t="s">
         <v>157</v>
       </c>
-      <c r="P277" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="278" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="278" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G278" t="s">
         <v>146</v>
       </c>
+      <c r="I278" t="s">
+        <v>150</v>
+      </c>
       <c r="J278" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K278" t="s">
         <v>131</v>
       </c>
       <c r="L278" t="s">
-        <v>162</v>
-      </c>
-      <c r="M278">
+        <v>161</v>
+      </c>
+      <c r="M278" s="13">
+        <f>M274</f>
         <v>35</v>
       </c>
       <c r="N278" t="s">
@@ -5878,25 +5877,26 @@
       <c r="O278" t="s">
         <v>157</v>
       </c>
-      <c r="P278" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="279" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G279" t="s">
         <v>146</v>
       </c>
+      <c r="I279" t="s">
+        <v>150</v>
+      </c>
       <c r="J279" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K279" t="s">
         <v>131</v>
       </c>
       <c r="L279" t="s">
-        <v>162</v>
-      </c>
-      <c r="M279">
-        <v>44</v>
+        <v>161</v>
+      </c>
+      <c r="M279" s="13">
+        <f>M275</f>
+        <v>48</v>
       </c>
       <c r="N279" t="s">
         <v>132</v>
@@ -5904,309 +5904,786 @@
       <c r="O279" t="s">
         <v>157</v>
       </c>
-      <c r="P279" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="280" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G280" t="s">
-        <v>151</v>
-      </c>
-      <c r="H280" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="I280" t="s">
+        <v>150</v>
       </c>
       <c r="J280" t="s">
-        <v>154</v>
+        <v>201</v>
       </c>
       <c r="K280" t="s">
         <v>131</v>
       </c>
       <c r="L280" t="s">
-        <v>162</v>
-      </c>
-      <c r="M280">
-        <v>41</v>
+        <v>161</v>
+      </c>
+      <c r="M280" s="13">
+        <f>M276</f>
+        <v>30</v>
       </c>
       <c r="N280" t="s">
         <v>132</v>
       </c>
-      <c r="P280" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O280" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="281" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G281" t="s">
-        <v>151</v>
-      </c>
-      <c r="H281" t="s">
+        <v>146</v>
+      </c>
+      <c r="I281" t="s">
+        <v>148</v>
+      </c>
+      <c r="J281" t="s">
         <v>152</v>
-      </c>
-      <c r="J281" t="s">
-        <v>155</v>
       </c>
       <c r="K281" t="s">
         <v>131</v>
       </c>
       <c r="L281" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M281">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="N281" t="s">
         <v>132</v>
       </c>
       <c r="P281" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="283" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A283" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="B283" s="7"/>
-    </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A285" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B285" s="2"/>
-      <c r="C285" s="2"/>
-      <c r="D285" s="2"/>
-      <c r="E285" s="2"/>
-      <c r="F285" s="2"/>
-      <c r="G285" s="2"/>
-      <c r="H285" s="2"/>
-      <c r="I285" s="2"/>
-      <c r="J285" s="2"/>
-      <c r="K285" s="2"/>
-      <c r="L285" s="2"/>
-      <c r="M285" s="2"/>
-      <c r="N285" s="2"/>
-      <c r="O285" s="2"/>
-      <c r="P285" s="2"/>
-    </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="282" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G282" t="s">
+        <v>146</v>
+      </c>
+      <c r="I282" t="s">
+        <v>148</v>
+      </c>
+      <c r="J282" t="s">
+        <v>153</v>
+      </c>
+      <c r="K282" t="s">
+        <v>131</v>
+      </c>
+      <c r="L282" t="s">
+        <v>161</v>
+      </c>
+      <c r="M282">
+        <v>34</v>
+      </c>
+      <c r="N282" t="s">
+        <v>132</v>
+      </c>
+      <c r="P282" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="283" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G283" t="s">
+        <v>146</v>
+      </c>
+      <c r="I283" t="s">
+        <v>148</v>
+      </c>
+      <c r="J283" t="s">
+        <v>154</v>
+      </c>
+      <c r="K283" t="s">
+        <v>131</v>
+      </c>
+      <c r="L283" t="s">
+        <v>161</v>
+      </c>
+      <c r="M283">
+        <v>46</v>
+      </c>
+      <c r="N283" t="s">
+        <v>132</v>
+      </c>
+      <c r="P283" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="284" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G284" t="s">
+        <v>146</v>
+      </c>
+      <c r="I284" t="s">
+        <v>148</v>
+      </c>
+      <c r="J284" t="s">
+        <v>201</v>
+      </c>
+      <c r="K284" t="s">
+        <v>131</v>
+      </c>
+      <c r="L284" t="s">
+        <v>161</v>
+      </c>
+      <c r="M284">
+        <v>29</v>
+      </c>
+      <c r="N284" t="s">
+        <v>132</v>
+      </c>
+      <c r="P284" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="285" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G285" t="s">
+        <v>146</v>
+      </c>
+      <c r="I285" t="s">
+        <v>149</v>
+      </c>
+      <c r="J285" t="s">
+        <v>152</v>
+      </c>
+      <c r="K285" t="s">
+        <v>131</v>
+      </c>
+      <c r="L285" t="s">
+        <v>161</v>
+      </c>
+      <c r="M285">
+        <v>29</v>
+      </c>
+      <c r="N285" t="s">
+        <v>132</v>
+      </c>
+      <c r="P285" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="286" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G286" t="s">
+        <v>146</v>
+      </c>
+      <c r="I286" t="s">
+        <v>149</v>
+      </c>
+      <c r="J286" t="s">
+        <v>153</v>
+      </c>
+      <c r="K286" t="s">
+        <v>131</v>
+      </c>
+      <c r="L286" t="s">
+        <v>161</v>
+      </c>
+      <c r="M286">
+        <v>35</v>
+      </c>
+      <c r="N286" t="s">
+        <v>132</v>
+      </c>
+      <c r="P286" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="287" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G287" t="s">
+        <v>146</v>
+      </c>
+      <c r="I287" t="s">
+        <v>149</v>
+      </c>
+      <c r="J287" t="s">
+        <v>154</v>
+      </c>
       <c r="K287" t="s">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="L287" t="s">
-        <v>182</v>
+        <v>161</v>
       </c>
       <c r="M287">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="N287" t="s">
-        <v>127</v>
-      </c>
-      <c r="O287" t="s">
-        <v>177</v>
+        <v>132</v>
       </c>
       <c r="P287" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="288" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G288" t="s">
+        <v>146</v>
+      </c>
+      <c r="I288" t="s">
+        <v>149</v>
+      </c>
+      <c r="J288" t="s">
+        <v>201</v>
+      </c>
       <c r="K288" t="s">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="L288" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="M288">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="N288" t="s">
-        <v>127</v>
-      </c>
-      <c r="O288" t="s">
-        <v>179</v>
+        <v>132</v>
       </c>
       <c r="P288" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="289" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G289" t="s">
+        <v>146</v>
+      </c>
+      <c r="J289" t="s">
+        <v>152</v>
+      </c>
+      <c r="K289" t="s">
+        <v>131</v>
+      </c>
+      <c r="L289" t="s">
+        <v>161</v>
+      </c>
+      <c r="M289">
+        <v>29</v>
+      </c>
+      <c r="N289" t="s">
+        <v>132</v>
+      </c>
+      <c r="O289" t="s">
+        <v>156</v>
+      </c>
+      <c r="P289" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="290" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G290" t="s">
+        <v>146</v>
+      </c>
+      <c r="J290" t="s">
+        <v>153</v>
+      </c>
+      <c r="K290" t="s">
+        <v>131</v>
+      </c>
+      <c r="L290" t="s">
+        <v>161</v>
+      </c>
+      <c r="M290">
+        <v>35</v>
+      </c>
+      <c r="N290" t="s">
+        <v>132</v>
+      </c>
+      <c r="O290" t="s">
+        <v>156</v>
+      </c>
+      <c r="P290" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="291" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G291" t="s">
+        <v>146</v>
+      </c>
+      <c r="J291" t="s">
+        <v>154</v>
+      </c>
+      <c r="K291" t="s">
+        <v>131</v>
+      </c>
+      <c r="L291" t="s">
+        <v>161</v>
+      </c>
+      <c r="M291">
+        <v>44</v>
+      </c>
+      <c r="N291" t="s">
+        <v>132</v>
+      </c>
+      <c r="O291" t="s">
+        <v>156</v>
+      </c>
+      <c r="P291" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="292" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G292" t="s">
+        <v>146</v>
+      </c>
+      <c r="J292" t="s">
+        <v>201</v>
+      </c>
+      <c r="K292" t="s">
+        <v>131</v>
+      </c>
+      <c r="L292" t="s">
+        <v>161</v>
+      </c>
+      <c r="M292">
+        <v>29</v>
+      </c>
+      <c r="N292" t="s">
+        <v>132</v>
+      </c>
+      <c r="O292" t="s">
+        <v>156</v>
+      </c>
+      <c r="P292" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="293" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G293" t="s">
+        <v>151</v>
+      </c>
+      <c r="J293" t="s">
+        <v>152</v>
+      </c>
+      <c r="K293" t="s">
+        <v>131</v>
+      </c>
+      <c r="L293" t="s">
+        <v>161</v>
+      </c>
+      <c r="M293">
+        <v>29</v>
+      </c>
+      <c r="N293" t="s">
+        <v>132</v>
+      </c>
+      <c r="P293" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="294" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G294" t="s">
+        <v>151</v>
+      </c>
+      <c r="J294" t="s">
+        <v>153</v>
+      </c>
+      <c r="K294" t="s">
+        <v>131</v>
+      </c>
+      <c r="L294" t="s">
+        <v>161</v>
+      </c>
+      <c r="M294">
+        <v>40</v>
+      </c>
+      <c r="N294" t="s">
+        <v>132</v>
+      </c>
+      <c r="P294" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="295" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G295" t="s">
+        <v>151</v>
+      </c>
+      <c r="J295" t="s">
+        <v>154</v>
+      </c>
+      <c r="K295" t="s">
+        <v>131</v>
+      </c>
+      <c r="L295" t="s">
+        <v>161</v>
+      </c>
+      <c r="M295">
+        <v>56</v>
+      </c>
+      <c r="N295" t="s">
+        <v>132</v>
+      </c>
+      <c r="P295" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="296" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G296" t="s">
+        <v>151</v>
+      </c>
+      <c r="I296" t="s">
+        <v>204</v>
+      </c>
+      <c r="J296" t="s">
+        <v>152</v>
+      </c>
+      <c r="K296" t="s">
+        <v>131</v>
+      </c>
+      <c r="L296" t="s">
+        <v>161</v>
+      </c>
+      <c r="M296">
+        <v>30</v>
+      </c>
+      <c r="N296" t="s">
+        <v>132</v>
+      </c>
+      <c r="P296" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="297" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G297" t="s">
+        <v>151</v>
+      </c>
+      <c r="I297" t="s">
+        <v>204</v>
+      </c>
+      <c r="J297" t="s">
+        <v>153</v>
+      </c>
+      <c r="K297" t="s">
+        <v>131</v>
+      </c>
+      <c r="L297" t="s">
+        <v>161</v>
+      </c>
+      <c r="M297">
+        <v>41</v>
+      </c>
+      <c r="N297" t="s">
+        <v>132</v>
+      </c>
+      <c r="P297" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="298" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G298" t="s">
+        <v>151</v>
+      </c>
+      <c r="I298" t="s">
+        <v>204</v>
+      </c>
+      <c r="J298" t="s">
+        <v>154</v>
+      </c>
+      <c r="K298" t="s">
+        <v>131</v>
+      </c>
+      <c r="L298" t="s">
+        <v>161</v>
+      </c>
+      <c r="M298">
+        <v>56</v>
+      </c>
+      <c r="N298" t="s">
+        <v>132</v>
+      </c>
+      <c r="P298" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="299" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G299" t="s">
+        <v>151</v>
+      </c>
+      <c r="I299" t="s">
+        <v>205</v>
+      </c>
+      <c r="J299" t="s">
+        <v>153</v>
+      </c>
+      <c r="K299" t="s">
+        <v>131</v>
+      </c>
+      <c r="L299" t="s">
+        <v>161</v>
+      </c>
+      <c r="M299">
+        <v>41</v>
+      </c>
+      <c r="N299" t="s">
+        <v>132</v>
+      </c>
+      <c r="P299" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="300" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G300" t="s">
+        <v>151</v>
+      </c>
+      <c r="I300" t="s">
+        <v>205</v>
+      </c>
+      <c r="J300" t="s">
+        <v>154</v>
+      </c>
+      <c r="K300" t="s">
+        <v>131</v>
+      </c>
+      <c r="L300" t="s">
+        <v>161</v>
+      </c>
+      <c r="M300">
+        <v>41</v>
+      </c>
+      <c r="N300" t="s">
+        <v>132</v>
+      </c>
+      <c r="P300" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="302" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A302" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B302" s="2"/>
+      <c r="C302" s="2"/>
+      <c r="D302" s="2"/>
+      <c r="E302" s="2"/>
+      <c r="F302" s="2"/>
+      <c r="G302" s="2"/>
+      <c r="H302" s="2"/>
+      <c r="I302" s="2"/>
+      <c r="J302" s="2"/>
+      <c r="K302" s="2"/>
+      <c r="L302" s="2"/>
+      <c r="M302" s="2"/>
+      <c r="N302" s="2"/>
+      <c r="O302" s="2"/>
+      <c r="P302" s="2"/>
+    </row>
+    <row r="304" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="K304" t="s">
+        <v>169</v>
+      </c>
+      <c r="L304" t="s">
+        <v>180</v>
+      </c>
+      <c r="M304">
+        <v>1</v>
+      </c>
+      <c r="N304" t="s">
+        <v>127</v>
+      </c>
+      <c r="O304" t="s">
+        <v>176</v>
+      </c>
+      <c r="P304" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="305" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="K305" t="s">
+        <v>169</v>
+      </c>
+      <c r="L305" t="s">
+        <v>182</v>
+      </c>
+      <c r="M305">
+        <v>1</v>
+      </c>
+      <c r="N305" t="s">
+        <v>127</v>
+      </c>
+      <c r="O305" t="s">
+        <v>177</v>
+      </c>
+      <c r="P305" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="306" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G306" t="s">
         <v>140</v>
       </c>
-      <c r="J289" t="s">
+      <c r="J306" t="s">
+        <v>170</v>
+      </c>
+      <c r="K306" t="s">
+        <v>169</v>
+      </c>
+      <c r="L306" t="s">
+        <v>182</v>
+      </c>
+      <c r="M306">
+        <v>2</v>
+      </c>
+      <c r="N306" t="s">
+        <v>127</v>
+      </c>
+      <c r="O306" t="s">
+        <v>173</v>
+      </c>
+      <c r="P306" t="s">
         <v>171</v>
       </c>
-      <c r="K289" t="s">
+    </row>
+    <row r="307" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J307" t="s">
         <v>170</v>
       </c>
-      <c r="L289" t="s">
+      <c r="K307" t="s">
+        <v>169</v>
+      </c>
+      <c r="L307" t="s">
+        <v>182</v>
+      </c>
+      <c r="M307">
+        <v>1</v>
+      </c>
+      <c r="N307" t="s">
+        <v>127</v>
+      </c>
+      <c r="O307" t="s">
+        <v>174</v>
+      </c>
+      <c r="P307" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="308" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="K308" t="s">
+        <v>169</v>
+      </c>
+      <c r="L308" t="s">
+        <v>181</v>
+      </c>
+      <c r="M308">
+        <v>1</v>
+      </c>
+      <c r="N308" t="s">
+        <v>127</v>
+      </c>
+      <c r="O308" t="s">
         <v>184</v>
       </c>
-      <c r="M289">
-        <v>2</v>
-      </c>
-      <c r="N289" t="s">
+      <c r="P308" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="309" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="K309" t="s">
+        <v>169</v>
+      </c>
+      <c r="L309" t="s">
+        <v>183</v>
+      </c>
+      <c r="M309">
+        <v>1</v>
+      </c>
+      <c r="N309" t="s">
         <v>127</v>
       </c>
-      <c r="O289" t="s">
-        <v>174</v>
-      </c>
-      <c r="P289" t="s">
+      <c r="O309" t="s">
+        <v>175</v>
+      </c>
+      <c r="P309" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="J290" t="s">
-        <v>171</v>
-      </c>
-      <c r="K290" t="s">
-        <v>170</v>
-      </c>
-      <c r="L290" t="s">
-        <v>184</v>
-      </c>
-      <c r="M290">
-        <v>1</v>
-      </c>
-      <c r="N290" t="s">
-        <v>127</v>
-      </c>
-      <c r="O290" t="s">
-        <v>175</v>
-      </c>
-      <c r="P290" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K291" t="s">
-        <v>170</v>
-      </c>
-      <c r="L291" t="s">
-        <v>183</v>
-      </c>
-      <c r="M291">
-        <v>1</v>
-      </c>
-      <c r="N291" t="s">
-        <v>127</v>
-      </c>
-      <c r="O291" t="s">
-        <v>186</v>
-      </c>
-      <c r="P291" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K292" t="s">
-        <v>170</v>
-      </c>
-      <c r="L292" t="s">
-        <v>185</v>
-      </c>
-      <c r="M292">
-        <v>1</v>
-      </c>
-      <c r="N292" t="s">
-        <v>127</v>
-      </c>
-      <c r="O292" t="s">
-        <v>176</v>
-      </c>
-      <c r="P292" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="294" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K294" t="s">
-        <v>170</v>
-      </c>
-      <c r="L294" t="s">
-        <v>189</v>
-      </c>
-      <c r="M294">
+    <row r="311" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="K311" t="s">
+        <v>169</v>
+      </c>
+      <c r="L311" t="s">
+        <v>187</v>
+      </c>
+      <c r="M311">
         <v>13</v>
       </c>
-      <c r="N294" t="s">
+      <c r="N311" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="313" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A313" s="2" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A296" s="2" t="s">
+      <c r="B313" s="2"/>
+      <c r="C313" s="2"/>
+      <c r="D313" s="2"/>
+      <c r="E313" s="2"/>
+      <c r="F313" s="2"/>
+      <c r="G313" s="2"/>
+      <c r="H313" s="2"/>
+      <c r="I313" s="2"/>
+      <c r="J313" s="2"/>
+      <c r="K313" s="2"/>
+      <c r="L313" s="2"/>
+      <c r="M313" s="2"/>
+      <c r="N313" s="2"/>
+      <c r="O313" s="2"/>
+      <c r="P313" s="2"/>
+    </row>
+    <row r="315" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B315" t="s">
+        <v>196</v>
+      </c>
+      <c r="K315" t="s">
+        <v>194</v>
+      </c>
+      <c r="L315" t="s">
+        <v>191</v>
+      </c>
+      <c r="M315">
+        <v>0.24</v>
+      </c>
+      <c r="N315" t="s">
+        <v>193</v>
+      </c>
+      <c r="P315" t="s">
         <v>192</v>
       </c>
-      <c r="B296" s="2"/>
-      <c r="C296" s="2"/>
-      <c r="D296" s="2"/>
-      <c r="E296" s="2"/>
-      <c r="F296" s="2"/>
-      <c r="G296" s="2"/>
-      <c r="H296" s="2"/>
-      <c r="I296" s="2"/>
-      <c r="J296" s="2"/>
-      <c r="K296" s="2"/>
-      <c r="L296" s="2"/>
-      <c r="M296" s="2"/>
-      <c r="N296" s="2"/>
-      <c r="O296" s="2"/>
-      <c r="P296" s="2"/>
-    </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B298" t="s">
+    </row>
+    <row r="316" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B316" t="s">
+        <v>197</v>
+      </c>
+      <c r="K316" t="s">
+        <v>194</v>
+      </c>
+      <c r="L316" t="s">
+        <v>191</v>
+      </c>
+      <c r="M316">
+        <v>0.24</v>
+      </c>
+      <c r="N316" t="s">
+        <v>193</v>
+      </c>
+      <c r="P316" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="317" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B317" t="s">
         <v>198</v>
       </c>
-      <c r="K298" t="s">
-        <v>196</v>
-      </c>
-      <c r="L298" t="s">
+      <c r="K317" t="s">
+        <v>194</v>
+      </c>
+      <c r="L317" t="s">
+        <v>191</v>
+      </c>
+      <c r="M317">
+        <v>0</v>
+      </c>
+      <c r="N317" t="s">
         <v>193</v>
       </c>
-      <c r="M298">
-        <v>0.24</v>
-      </c>
-      <c r="N298" t="s">
-        <v>195</v>
-      </c>
-      <c r="P298" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B299" t="s">
+      <c r="O317" t="s">
         <v>199</v>
-      </c>
-      <c r="K299" t="s">
-        <v>196</v>
-      </c>
-      <c r="L299" t="s">
-        <v>193</v>
-      </c>
-      <c r="M299">
-        <v>0.24</v>
-      </c>
-      <c r="N299" t="s">
-        <v>195</v>
-      </c>
-      <c r="P299" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="300" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B300" t="s">
-        <v>200</v>
-      </c>
-      <c r="K300" t="s">
-        <v>196</v>
-      </c>
-      <c r="L300" t="s">
-        <v>193</v>
-      </c>
-      <c r="M300">
-        <v>0</v>
-      </c>
-      <c r="N300" t="s">
-        <v>195</v>
-      </c>
-      <c r="O300" t="s">
-        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed to 10% clover in conv. leys for N-req calc.
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -934,9 +934,6 @@
     <t>grass clover ley (40% clover) and three harvest</t>
   </si>
   <si>
-    <t>grass clover ley (20% clover) and three harvest</t>
-  </si>
-  <si>
     <t>grass ley and three harvest</t>
   </si>
   <si>
@@ -962,6 +959,9 @@
   </si>
   <si>
     <t>Minimum share of total N from manure on area where manure is applied</t>
+  </si>
+  <si>
+    <t>grass clover ley (10% clover) and three harvest</t>
   </si>
 </sst>
 </file>
@@ -1739,7 +1739,7 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1763,7 +1763,7 @@
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="P21" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="Q21">
         <v>66</v>
@@ -1772,10 +1772,10 @@
         <v>103</v>
       </c>
       <c r="S21" t="s">
+        <v>309</v>
+      </c>
+      <c r="T21" t="s">
         <v>310</v>
-      </c>
-      <c r="T21" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="23" spans="1:20" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3780,10 +3780,10 @@
         <v>11</v>
       </c>
       <c r="Q150">
-        <v>15</v>
+        <v>18.5</v>
       </c>
       <c r="S150" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
     </row>
     <row r="151" spans="1:20" x14ac:dyDescent="0.25">
@@ -3808,7 +3808,7 @@
         <v>12</v>
       </c>
       <c r="Q151">
-        <v>20</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="152" spans="1:20" x14ac:dyDescent="0.25">
@@ -4817,7 +4817,7 @@
         <v>4.2</v>
       </c>
       <c r="T193" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="194" spans="1:20" x14ac:dyDescent="0.25">
@@ -4842,7 +4842,7 @@
         <v>3.3</v>
       </c>
       <c r="T194" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="195" spans="1:20" x14ac:dyDescent="0.25">
@@ -4868,7 +4868,7 @@
         <v>3.75</v>
       </c>
       <c r="S195" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="196" spans="1:20" x14ac:dyDescent="0.25">
@@ -5010,7 +5010,7 @@
         <v>20</v>
       </c>
       <c r="S201" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="202" spans="1:20" x14ac:dyDescent="0.25">
@@ -7098,7 +7098,7 @@
         <v>3</v>
       </c>
       <c r="S332" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="333" spans="1:19" x14ac:dyDescent="0.25">
@@ -7229,7 +7229,7 @@
         <v>3</v>
       </c>
       <c r="S340" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="341" spans="1:19" x14ac:dyDescent="0.25">
@@ -7677,7 +7677,7 @@
         <v>3</v>
       </c>
       <c r="S373" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="374" spans="1:19" x14ac:dyDescent="0.25">
@@ -8979,7 +8979,7 @@
         <v>0.6</v>
       </c>
       <c r="T477" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="478" spans="1:20" x14ac:dyDescent="0.25">
@@ -8994,7 +8994,7 @@
         <v>1.6</v>
       </c>
       <c r="T478" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="479" spans="1:20" x14ac:dyDescent="0.25">
@@ -9010,7 +9010,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="S479" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="480" spans="1:20" x14ac:dyDescent="0.25">
@@ -10314,7 +10314,7 @@
         <v>5</v>
       </c>
       <c r="S570" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="571" spans="1:19" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>5</v>
       </c>
       <c r="S576" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="577" spans="1:17" x14ac:dyDescent="0.25">
@@ -10830,7 +10830,7 @@
         <v>10</v>
       </c>
       <c r="S607" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="608" spans="1:19" x14ac:dyDescent="0.25">
@@ -11970,7 +11970,7 @@
         <v>5.6</v>
       </c>
       <c r="T700" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="701" spans="1:20" x14ac:dyDescent="0.25">
@@ -11985,7 +11985,7 @@
         <v>3</v>
       </c>
       <c r="T701" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="702" spans="1:20" x14ac:dyDescent="0.25">
@@ -12001,7 +12001,7 @@
         <v>4.3</v>
       </c>
       <c r="S702" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="703" spans="1:20" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Removed N2O emissions from semi-natural grasslands on organic soils which seems to be the case in NIR although a bit unclear
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2484" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2489" uniqueCount="316">
   <si>
     <t>f_crop</t>
   </si>
@@ -965,6 +965,9 @@
   </si>
   <si>
     <t>Set to match K/ha in stat.</t>
+  </si>
+  <si>
+    <t>zero for all non-cropland</t>
   </si>
 </sst>
 </file>
@@ -1425,7 +1428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T794"/>
+  <dimension ref="A1:T795"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="21" customWidth="1"/>
@@ -13871,62 +13874,62 @@
         <v>174</v>
       </c>
       <c r="Q788">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="R788" t="s">
         <v>175</v>
       </c>
-      <c r="T788" t="s">
+      <c r="S788" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="789" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C789" t="s">
+        <v>183</v>
+      </c>
+      <c r="O789" t="s">
+        <v>156</v>
+      </c>
+      <c r="P789" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q789">
+        <v>13</v>
+      </c>
+      <c r="R789" t="s">
+        <v>175</v>
+      </c>
+      <c r="T789" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="790" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A790" s="2" t="s">
+    <row r="791" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A791" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B790" s="2"/>
-      <c r="C790" s="2"/>
-      <c r="D790" s="2"/>
-      <c r="E790" s="2"/>
-      <c r="F790" s="2"/>
-      <c r="G790" s="2"/>
-      <c r="H790" s="2"/>
-      <c r="I790" s="2"/>
-      <c r="J790" s="2"/>
-      <c r="K790" s="2"/>
-      <c r="L790" s="2"/>
-      <c r="M790" s="2"/>
-      <c r="N790" s="2"/>
-      <c r="O790" s="2"/>
-      <c r="P790" s="2"/>
-      <c r="Q790" s="2"/>
-      <c r="R790" s="2"/>
-      <c r="S790" s="2"/>
-      <c r="T790" s="2"/>
-    </row>
-    <row r="792" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="C792" t="s">
-        <v>183</v>
-      </c>
-      <c r="O792" t="s">
-        <v>181</v>
-      </c>
-      <c r="P792" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q792">
-        <v>0.24</v>
-      </c>
-      <c r="R792" t="s">
-        <v>180</v>
-      </c>
-      <c r="T792" t="s">
-        <v>179</v>
-      </c>
+      <c r="B791" s="2"/>
+      <c r="C791" s="2"/>
+      <c r="D791" s="2"/>
+      <c r="E791" s="2"/>
+      <c r="F791" s="2"/>
+      <c r="G791" s="2"/>
+      <c r="H791" s="2"/>
+      <c r="I791" s="2"/>
+      <c r="J791" s="2"/>
+      <c r="K791" s="2"/>
+      <c r="L791" s="2"/>
+      <c r="M791" s="2"/>
+      <c r="N791" s="2"/>
+      <c r="O791" s="2"/>
+      <c r="P791" s="2"/>
+      <c r="Q791" s="2"/>
+      <c r="R791" s="2"/>
+      <c r="S791" s="2"/>
+      <c r="T791" s="2"/>
     </row>
     <row r="793" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C793" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="O793" t="s">
         <v>181</v>
@@ -13946,7 +13949,7 @@
     </row>
     <row r="794" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C794" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O794" t="s">
         <v>181</v>
@@ -13955,12 +13958,32 @@
         <v>178</v>
       </c>
       <c r="Q794">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="R794" t="s">
         <v>180</v>
       </c>
-      <c r="S794" t="s">
+      <c r="T794" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="795" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C795" t="s">
+        <v>185</v>
+      </c>
+      <c r="O795" t="s">
+        <v>181</v>
+      </c>
+      <c r="P795" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q795">
+        <v>0</v>
+      </c>
+      <c r="R795" t="s">
+        <v>180</v>
+      </c>
+      <c r="S795" t="s">
         <v>186</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reduced clover % for organic ley + changed validation data for N input to organic areas
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -903,9 +903,6 @@
     <t>"Jordbruksverket (2023) Rekommendationer för gödsling och kalkning 2023"</t>
   </si>
   <si>
-    <t>grass clover ley (40% clover) and three harvest</t>
-  </si>
-  <si>
     <t>grass ley and three harvest</t>
   </si>
   <si>
@@ -1081,6 +1078,9 @@
   </si>
   <si>
     <t>Assume that some 'Fallow' is used as green manure</t>
+  </si>
+  <si>
+    <t>grass clover ley (avg. 20/40% clover) and three harvest</t>
   </si>
 </sst>
 </file>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>174</v>
@@ -1845,7 +1845,7 @@
         <v>98</v>
       </c>
       <c r="I15" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="R15" s="4" t="s">
         <v>211</v>
@@ -1857,7 +1857,7 @@
         <v>210</v>
       </c>
       <c r="U15" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
@@ -1899,7 +1899,7 @@
         <v>98</v>
       </c>
       <c r="I19" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="R19" s="4" t="s">
         <v>212</v>
@@ -1911,7 +1911,7 @@
         <v>213</v>
       </c>
       <c r="U19" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -1938,7 +1938,7 @@
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1964,7 +1964,7 @@
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="R24" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="S24">
         <v>66</v>
@@ -1973,10 +1973,10 @@
         <v>97</v>
       </c>
       <c r="U24" t="s">
+        <v>299</v>
+      </c>
+      <c r="V24" t="s">
         <v>300</v>
-      </c>
-      <c r="V24" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>18.5</v>
       </c>
       <c r="U153" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="154" spans="1:22" x14ac:dyDescent="0.25">
@@ -4058,10 +4058,10 @@
         <v>10</v>
       </c>
       <c r="S155">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="U155" t="s">
-        <v>294</v>
+        <v>353</v>
       </c>
     </row>
     <row r="156" spans="1:22" x14ac:dyDescent="0.25">
@@ -4088,7 +4088,7 @@
         <v>11</v>
       </c>
       <c r="S156">
-        <v>13</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="157" spans="1:22" x14ac:dyDescent="0.25">
@@ -5116,7 +5116,7 @@
         <v>4.2</v>
       </c>
       <c r="V196" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="197" spans="1:22" x14ac:dyDescent="0.25">
@@ -5143,7 +5143,7 @@
         <v>3.3</v>
       </c>
       <c r="V197" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="198" spans="1:22" x14ac:dyDescent="0.25">
@@ -5171,7 +5171,7 @@
         <v>3.75</v>
       </c>
       <c r="U198" s="6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="199" spans="1:22" x14ac:dyDescent="0.25">
@@ -5325,7 +5325,7 @@
         <v>20</v>
       </c>
       <c r="U204" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="205" spans="1:22" x14ac:dyDescent="0.25">
@@ -5917,10 +5917,10 @@
         <v>60</v>
       </c>
       <c r="U228" t="s">
+        <v>343</v>
+      </c>
+      <c r="V228" t="s">
         <v>344</v>
-      </c>
-      <c r="V228" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="229" spans="1:22" x14ac:dyDescent="0.25">
@@ -5939,7 +5939,7 @@
         <v>30</v>
       </c>
       <c r="U229" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="230" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -6017,19 +6017,19 @@
     </row>
     <row r="235" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A235" s="19" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B235" s="4"/>
     </row>
     <row r="236" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A236" s="19" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B236" s="4"/>
     </row>
     <row r="237" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A237" s="19" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B237" s="4"/>
     </row>
@@ -6046,7 +6046,7 @@
         <v>245</v>
       </c>
       <c r="U238" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="V238" t="s">
         <v>250</v>
@@ -7510,7 +7510,7 @@
         <v>3</v>
       </c>
       <c r="U338" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="339" spans="1:21" x14ac:dyDescent="0.25">
@@ -7657,7 +7657,7 @@
         <v>3</v>
       </c>
       <c r="U346" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="347" spans="1:21" x14ac:dyDescent="0.25">
@@ -8121,7 +8121,7 @@
         <v>3</v>
       </c>
       <c r="U379" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="380" spans="1:21" x14ac:dyDescent="0.25">
@@ -9469,7 +9469,7 @@
         <v>0.6</v>
       </c>
       <c r="V483" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="484" spans="1:22" x14ac:dyDescent="0.25">
@@ -9486,7 +9486,7 @@
         <v>1.6</v>
       </c>
       <c r="V484" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="485" spans="1:22" x14ac:dyDescent="0.25">
@@ -9504,7 +9504,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="U485" s="6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="486" spans="1:22" x14ac:dyDescent="0.25">
@@ -10871,7 +10871,7 @@
         <v>5</v>
       </c>
       <c r="U577" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="578" spans="1:21" x14ac:dyDescent="0.25">
@@ -10982,7 +10982,7 @@
         <v>5</v>
       </c>
       <c r="U583" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="584" spans="1:21" x14ac:dyDescent="0.25">
@@ -11412,7 +11412,7 @@
         <v>10</v>
       </c>
       <c r="U614" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="615" spans="1:21" x14ac:dyDescent="0.25">
@@ -12600,7 +12600,7 @@
         <v>5.6</v>
       </c>
       <c r="V707" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="708" spans="1:22" x14ac:dyDescent="0.25">
@@ -12617,7 +12617,7 @@
         <v>3</v>
       </c>
       <c r="V708" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="709" spans="1:22" x14ac:dyDescent="0.25">
@@ -12635,7 +12635,7 @@
         <v>4.3</v>
       </c>
       <c r="U709" s="6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="710" spans="1:22" x14ac:dyDescent="0.25">
@@ -12739,7 +12739,7 @@
       </c>
       <c r="T717" s="5"/>
       <c r="U717" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="719" spans="1:22" x14ac:dyDescent="0.25">
@@ -12787,7 +12787,7 @@
     </row>
     <row r="721" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A721" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B721" s="1"/>
       <c r="C721" s="1"/>
@@ -14503,7 +14503,7 @@
         <v>167</v>
       </c>
       <c r="U798" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="799" spans="1:22" x14ac:dyDescent="0.25">
@@ -14614,7 +14614,7 @@
     </row>
     <row r="807" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A807" s="27" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B807" s="27"/>
       <c r="C807" s="28"/>
@@ -14640,10 +14640,10 @@
     </row>
     <row r="809" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I809" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="R809" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="S809" s="11">
         <f>213/(213 + 60)*100</f>
@@ -14653,15 +14653,15 @@
         <v>97</v>
       </c>
       <c r="V809" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="810" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I810" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="R810" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="S810" s="11">
         <f>60/(213 + 60)*100</f>
@@ -14671,15 +14671,15 @@
         <v>97</v>
       </c>
       <c r="V810" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="812" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I812" t="s">
+        <v>326</v>
+      </c>
+      <c r="R812" t="s">
         <v>327</v>
-      </c>
-      <c r="R812" t="s">
-        <v>328</v>
       </c>
       <c r="S812">
         <v>45</v>
@@ -14688,15 +14688,15 @@
         <v>97</v>
       </c>
       <c r="V812" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="813" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I813" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="R813" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="S813">
         <v>48</v>
@@ -14705,25 +14705,25 @@
         <v>97</v>
       </c>
       <c r="V813" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="815" spans="1:22" x14ac:dyDescent="0.25">
       <c r="R815" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S815" s="30">
         <f>S822</f>
         <v>-5.9999999999999995E-4</v>
       </c>
       <c r="T815" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="U815" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="V815" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="816" spans="1:22" x14ac:dyDescent="0.25">
@@ -14734,20 +14734,20 @@
         <v>142</v>
       </c>
       <c r="R816" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S816" s="29">
         <f>-(45.5*0.1+10.7*0.9)/1000</f>
         <v>-1.418E-2</v>
       </c>
       <c r="T816" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="U816" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="V816" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="817" spans="1:22" x14ac:dyDescent="0.25">
@@ -14758,14 +14758,14 @@
         <v>142</v>
       </c>
       <c r="R817" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S817" s="33">
         <f>S816</f>
         <v>-1.418E-2</v>
       </c>
       <c r="T817" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="818" spans="1:22" x14ac:dyDescent="0.25">
@@ -14776,20 +14776,20 @@
         <v>98</v>
       </c>
       <c r="R818" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S818" s="29">
         <f>-(45.5*0.4+10.7*0.6)/1000</f>
         <v>-2.4619999999999996E-2</v>
       </c>
       <c r="T818" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="U818" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="V818" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="819" spans="1:22" x14ac:dyDescent="0.25">
@@ -14800,14 +14800,14 @@
         <v>98</v>
       </c>
       <c r="R819" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S819" s="33">
         <f>S818</f>
         <v>-2.4619999999999996E-2</v>
       </c>
       <c r="T819" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="820" spans="1:22" x14ac:dyDescent="0.25">
@@ -14816,20 +14816,20 @@
       </c>
       <c r="B820" s="4"/>
       <c r="R820" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S820" s="4">
         <f>-10.7/1000</f>
         <v>-1.0699999999999999E-2</v>
       </c>
       <c r="T820" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="U820" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="V820" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="821" spans="1:22" x14ac:dyDescent="0.25">
@@ -14838,20 +14838,20 @@
       </c>
       <c r="B821" s="4"/>
       <c r="R821" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S821" s="4">
         <f>-10.7/1000</f>
         <v>-1.0699999999999999E-2</v>
       </c>
       <c r="T821" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="U821" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="V821" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="822" spans="1:22" x14ac:dyDescent="0.25">
@@ -14859,56 +14859,56 @@
         <v>226</v>
       </c>
       <c r="R822" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S822">
         <f>-0.6/1000</f>
         <v>-5.9999999999999995E-4</v>
       </c>
       <c r="T822" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="V822" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="823" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B823" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="R823" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S823" s="29">
         <f>-20*0.45/0.85/1000</f>
         <v>-1.0588235294117647E-2</v>
       </c>
       <c r="T823" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="U823" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="V823" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="825" spans="1:22" x14ac:dyDescent="0.25">
       <c r="D825" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="R825" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="S825">
         <f>-9.2/1000</f>
         <v>-9.1999999999999998E-3</v>
       </c>
       <c r="T825" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="V825" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="827" spans="1:22" x14ac:dyDescent="0.25">
@@ -14916,16 +14916,16 @@
         <v>107</v>
       </c>
       <c r="R827" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="S827" s="31">
         <v>-0.5</v>
       </c>
       <c r="T827" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="V827" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="828" spans="1:22" x14ac:dyDescent="0.25">
@@ -14933,16 +14933,16 @@
         <v>108</v>
       </c>
       <c r="R828" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="S828" s="31">
         <v>-1</v>
       </c>
       <c r="T828" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="V828" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="829" spans="1:22" x14ac:dyDescent="0.25">
@@ -14950,106 +14950,106 @@
         <v>208</v>
       </c>
       <c r="R829" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="S829" s="22">
         <v>-1</v>
       </c>
       <c r="T829" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="U829" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="830" spans="1:22" x14ac:dyDescent="0.25">
       <c r="R830" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="S830" s="22">
         <f>-0.4 / ( (2*30.97) / (2*30.97 + 5*16) )</f>
         <v>-0.91662899580238943</v>
       </c>
       <c r="T830" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="U830" s="32" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="V830" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="831" spans="1:22" x14ac:dyDescent="0.25">
       <c r="R831" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="S831" s="22">
         <f>0.6 / ( (2*39.1) / (2*39.1 + 16) )</f>
         <v>0.72276214833759589</v>
       </c>
       <c r="T831" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="U831" s="32" t="s">
+        <v>335</v>
+      </c>
+      <c r="V831" t="s">
         <v>336</v>
-      </c>
-      <c r="V831" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="833" spans="9:22" x14ac:dyDescent="0.25">
       <c r="R833" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="S833" s="31">
         <f>3/5</f>
         <v>0.6</v>
       </c>
       <c r="T833" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="U833" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="V833" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="835" spans="9:22" x14ac:dyDescent="0.25">
       <c r="I835" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="Q835" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R835" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="S835" s="31">
         <f>0.12*(44/12)</f>
         <v>0.43999999999999995</v>
       </c>
       <c r="T835" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="836" spans="9:22" x14ac:dyDescent="0.25">
       <c r="I836" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="Q836" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R836" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="S836" s="31">
         <f>0.13*(44/12)</f>
         <v>0.47666666666666668</v>
       </c>
       <c r="T836" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="837" spans="9:22" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated shares organic soils to only include 'peat' and added N2O factor for semi-natural grasslands on organic soils
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2502" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2507" uniqueCount="355">
   <si>
     <t>f_crop</t>
   </si>
@@ -936,9 +936,6 @@
     <t>Set to match K/ha in stat.</t>
   </si>
   <si>
-    <t>zero for all non-cropland</t>
-  </si>
-  <si>
     <t>Liming</t>
   </si>
   <si>
@@ -1081,6 +1078,12 @@
   </si>
   <si>
     <t>grass clover ley (avg. 20/40% clover) and three harvest</t>
+  </si>
+  <si>
+    <t>Not included in NIR, reported under forest</t>
+  </si>
+  <si>
+    <t>Pers. comm. Mattias Lindblad (2024-11-14)</t>
   </si>
 </sst>
 </file>
@@ -1555,7 +1558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V837"/>
+  <dimension ref="A1:V838"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="21" customWidth="1"/>
@@ -1580,13 +1583,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>174</v>
@@ -1845,7 +1848,7 @@
         <v>98</v>
       </c>
       <c r="I15" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="R15" s="4" t="s">
         <v>211</v>
@@ -1857,7 +1860,7 @@
         <v>210</v>
       </c>
       <c r="U15" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
@@ -1899,7 +1902,7 @@
         <v>98</v>
       </c>
       <c r="I19" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="R19" s="4" t="s">
         <v>212</v>
@@ -1911,7 +1914,7 @@
         <v>213</v>
       </c>
       <c r="U19" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -4061,7 +4064,7 @@
         <v>12</v>
       </c>
       <c r="U155" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="156" spans="1:22" x14ac:dyDescent="0.25">
@@ -5917,10 +5920,10 @@
         <v>60</v>
       </c>
       <c r="U228" t="s">
+        <v>342</v>
+      </c>
+      <c r="V228" t="s">
         <v>343</v>
-      </c>
-      <c r="V228" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="229" spans="1:22" x14ac:dyDescent="0.25">
@@ -5939,7 +5942,7 @@
         <v>30</v>
       </c>
       <c r="U229" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="230" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -6017,19 +6020,19 @@
     </row>
     <row r="235" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A235" s="19" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B235" s="4"/>
     </row>
     <row r="236" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A236" s="19" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B236" s="4"/>
     </row>
     <row r="237" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A237" s="19" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B237" s="4"/>
     </row>
@@ -6046,7 +6049,7 @@
         <v>245</v>
       </c>
       <c r="U238" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="V238" t="s">
         <v>250</v>
@@ -12787,7 +12790,7 @@
     </row>
     <row r="721" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A721" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B721" s="1"/>
       <c r="C721" s="1"/>
@@ -14502,9 +14505,6 @@
       <c r="T798" t="s">
         <v>167</v>
       </c>
-      <c r="U798" t="s">
-        <v>305</v>
-      </c>
     </row>
     <row r="799" spans="1:22" x14ac:dyDescent="0.25">
       <c r="E799" t="s">
@@ -14526,55 +14526,58 @@
         <v>151</v>
       </c>
     </row>
-    <row r="801" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A801" s="2" t="s">
+    <row r="800" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E800" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q800" t="s">
+        <v>148</v>
+      </c>
+      <c r="R800" t="s">
+        <v>166</v>
+      </c>
+      <c r="S800">
+        <v>13</v>
+      </c>
+      <c r="T800" t="s">
+        <v>167</v>
+      </c>
+      <c r="U800" t="s">
+        <v>353</v>
+      </c>
+      <c r="V800" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="802" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A802" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B801" s="2"/>
-      <c r="C801" s="2"/>
-      <c r="D801" s="2"/>
-      <c r="E801" s="2"/>
-      <c r="F801" s="2"/>
-      <c r="G801" s="2"/>
-      <c r="H801" s="2"/>
-      <c r="I801" s="2"/>
-      <c r="J801" s="2"/>
-      <c r="K801" s="2"/>
-      <c r="L801" s="2"/>
-      <c r="M801" s="2"/>
-      <c r="N801" s="2"/>
-      <c r="O801" s="2"/>
-      <c r="P801" s="2"/>
-      <c r="Q801" s="2"/>
-      <c r="R801" s="2"/>
-      <c r="S801" s="2"/>
-      <c r="T801" s="2"/>
-      <c r="U801" s="2"/>
-      <c r="V801" s="2"/>
-    </row>
-    <row r="803" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="E803" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q803" t="s">
-        <v>173</v>
-      </c>
-      <c r="R803" t="s">
-        <v>170</v>
-      </c>
-      <c r="S803">
-        <v>0.24</v>
-      </c>
-      <c r="T803" t="s">
-        <v>172</v>
-      </c>
-      <c r="V803" t="s">
-        <v>171</v>
-      </c>
+      <c r="B802" s="2"/>
+      <c r="C802" s="2"/>
+      <c r="D802" s="2"/>
+      <c r="E802" s="2"/>
+      <c r="F802" s="2"/>
+      <c r="G802" s="2"/>
+      <c r="H802" s="2"/>
+      <c r="I802" s="2"/>
+      <c r="J802" s="2"/>
+      <c r="K802" s="2"/>
+      <c r="L802" s="2"/>
+      <c r="M802" s="2"/>
+      <c r="N802" s="2"/>
+      <c r="O802" s="2"/>
+      <c r="P802" s="2"/>
+      <c r="Q802" s="2"/>
+      <c r="R802" s="2"/>
+      <c r="S802" s="2"/>
+      <c r="T802" s="2"/>
+      <c r="U802" s="2"/>
+      <c r="V802" s="2"/>
     </row>
     <row r="804" spans="1:22" x14ac:dyDescent="0.25">
       <c r="E804" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q804" t="s">
         <v>173</v>
@@ -14594,7 +14597,7 @@
     </row>
     <row r="805" spans="1:22" x14ac:dyDescent="0.25">
       <c r="E805" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q805" t="s">
         <v>173</v>
@@ -14603,381 +14606,383 @@
         <v>170</v>
       </c>
       <c r="S805">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="T805" t="s">
         <v>172</v>
       </c>
-      <c r="U805" t="s">
+      <c r="V805" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="806" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E806" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q806" t="s">
+        <v>173</v>
+      </c>
+      <c r="R806" t="s">
+        <v>170</v>
+      </c>
+      <c r="S806">
+        <v>0</v>
+      </c>
+      <c r="T806" t="s">
+        <v>172</v>
+      </c>
+      <c r="U806" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="807" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A807" s="27" t="s">
-        <v>306</v>
-      </c>
-      <c r="B807" s="27"/>
-      <c r="C807" s="28"/>
-      <c r="D807" s="28"/>
-      <c r="E807" s="28"/>
-      <c r="F807" s="28"/>
-      <c r="G807" s="28"/>
-      <c r="H807" s="28"/>
-      <c r="I807" s="28"/>
-      <c r="J807" s="28"/>
-      <c r="K807" s="28"/>
-      <c r="L807" s="28"/>
-      <c r="M807" s="28"/>
-      <c r="N807" s="28"/>
-      <c r="O807" s="28"/>
-      <c r="P807" s="28"/>
-      <c r="Q807" s="28"/>
-      <c r="R807" s="28"/>
-      <c r="S807" s="28"/>
-      <c r="T807" s="28"/>
-      <c r="U807" s="28"/>
-      <c r="V807" s="28"/>
-    </row>
-    <row r="809" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I809" t="s">
-        <v>326</v>
-      </c>
-      <c r="R809" t="s">
-        <v>324</v>
-      </c>
-      <c r="S809" s="11">
+    <row r="808" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A808" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="B808" s="27"/>
+      <c r="C808" s="28"/>
+      <c r="D808" s="28"/>
+      <c r="E808" s="28"/>
+      <c r="F808" s="28"/>
+      <c r="G808" s="28"/>
+      <c r="H808" s="28"/>
+      <c r="I808" s="28"/>
+      <c r="J808" s="28"/>
+      <c r="K808" s="28"/>
+      <c r="L808" s="28"/>
+      <c r="M808" s="28"/>
+      <c r="N808" s="28"/>
+      <c r="O808" s="28"/>
+      <c r="P808" s="28"/>
+      <c r="Q808" s="28"/>
+      <c r="R808" s="28"/>
+      <c r="S808" s="28"/>
+      <c r="T808" s="28"/>
+      <c r="U808" s="28"/>
+      <c r="V808" s="28"/>
+    </row>
+    <row r="810" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I810" t="s">
+        <v>325</v>
+      </c>
+      <c r="R810" t="s">
+        <v>323</v>
+      </c>
+      <c r="S810" s="11">
         <f>213/(213 + 60)*100</f>
         <v>78.021978021978029</v>
       </c>
-      <c r="T809" t="s">
+      <c r="T810" t="s">
         <v>97</v>
       </c>
-      <c r="V809" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="810" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I810" t="s">
-        <v>340</v>
-      </c>
-      <c r="R810" t="s">
+      <c r="V810" t="s">
         <v>324</v>
       </c>
-      <c r="S810" s="11">
+    </row>
+    <row r="811" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I811" t="s">
+        <v>339</v>
+      </c>
+      <c r="R811" t="s">
+        <v>323</v>
+      </c>
+      <c r="S811" s="11">
         <f>60/(213 + 60)*100</f>
         <v>21.978021978021978</v>
       </c>
-      <c r="T810" t="s">
+      <c r="T811" t="s">
         <v>97</v>
       </c>
-      <c r="V810" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="812" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I812" t="s">
-        <v>326</v>
-      </c>
-      <c r="R812" t="s">
-        <v>327</v>
-      </c>
-      <c r="S812">
-        <v>45</v>
-      </c>
-      <c r="T812" t="s">
-        <v>97</v>
-      </c>
-      <c r="V812" t="s">
-        <v>328</v>
+      <c r="V811" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="813" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I813" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
       <c r="R813" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="S813">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="T813" t="s">
         <v>97</v>
       </c>
       <c r="V813" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="815" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R815" t="s">
-        <v>307</v>
-      </c>
-      <c r="S815" s="30">
-        <f>S822</f>
+        <v>327</v>
+      </c>
+    </row>
+    <row r="814" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I814" t="s">
+        <v>339</v>
+      </c>
+      <c r="R814" t="s">
+        <v>326</v>
+      </c>
+      <c r="S814">
+        <v>48</v>
+      </c>
+      <c r="T814" t="s">
+        <v>97</v>
+      </c>
+      <c r="V814" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="816" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R816" t="s">
+        <v>306</v>
+      </c>
+      <c r="S816" s="30">
+        <f>S823</f>
         <v>-5.9999999999999995E-4</v>
       </c>
-      <c r="T815" t="s">
-        <v>310</v>
-      </c>
-      <c r="U815" t="s">
-        <v>323</v>
-      </c>
-      <c r="V815" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="816" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A816" t="s">
+      <c r="T816" t="s">
+        <v>309</v>
+      </c>
+      <c r="U816" t="s">
+        <v>322</v>
+      </c>
+      <c r="V816" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="817" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A817" t="s">
         <v>37</v>
       </c>
-      <c r="G816" t="s">
+      <c r="G817" t="s">
         <v>142</v>
       </c>
-      <c r="R816" t="s">
-        <v>307</v>
-      </c>
-      <c r="S816" s="29">
+      <c r="R817" t="s">
+        <v>306</v>
+      </c>
+      <c r="S817" s="29">
         <f>-(45.5*0.1+10.7*0.9)/1000</f>
         <v>-1.418E-2</v>
       </c>
-      <c r="T816" t="s">
-        <v>310</v>
-      </c>
-      <c r="U816" t="s">
-        <v>341</v>
-      </c>
-      <c r="V816" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="817" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A817" t="s">
-        <v>38</v>
-      </c>
-      <c r="G817" t="s">
-        <v>142</v>
-      </c>
-      <c r="R817" t="s">
-        <v>307</v>
-      </c>
-      <c r="S817" s="33">
-        <f>S816</f>
-        <v>-1.418E-2</v>
-      </c>
       <c r="T817" t="s">
-        <v>310</v>
+        <v>309</v>
+      </c>
+      <c r="U817" t="s">
+        <v>340</v>
+      </c>
+      <c r="V817" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="818" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A818" t="s">
+        <v>38</v>
+      </c>
+      <c r="G818" t="s">
+        <v>142</v>
+      </c>
+      <c r="R818" t="s">
+        <v>306</v>
+      </c>
+      <c r="S818" s="33">
+        <f>S817</f>
+        <v>-1.418E-2</v>
+      </c>
+      <c r="T818" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="819" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A819" t="s">
         <v>37</v>
       </c>
-      <c r="G818" t="s">
+      <c r="G819" t="s">
         <v>98</v>
       </c>
-      <c r="R818" t="s">
-        <v>307</v>
-      </c>
-      <c r="S818" s="29">
+      <c r="R819" t="s">
+        <v>306</v>
+      </c>
+      <c r="S819" s="29">
         <f>-(45.5*0.4+10.7*0.6)/1000</f>
         <v>-2.4619999999999996E-2</v>
       </c>
-      <c r="T818" t="s">
-        <v>310</v>
-      </c>
-      <c r="U818" t="s">
-        <v>342</v>
-      </c>
-      <c r="V818" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="819" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A819" t="s">
+      <c r="T819" t="s">
+        <v>309</v>
+      </c>
+      <c r="U819" t="s">
+        <v>341</v>
+      </c>
+      <c r="V819" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="820" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A820" t="s">
         <v>38</v>
       </c>
-      <c r="G819" t="s">
+      <c r="G820" t="s">
         <v>98</v>
       </c>
-      <c r="R819" t="s">
-        <v>307</v>
-      </c>
-      <c r="S819" s="33">
-        <f>S818</f>
+      <c r="R820" t="s">
+        <v>306</v>
+      </c>
+      <c r="S820" s="33">
+        <f>S819</f>
         <v>-2.4619999999999996E-2</v>
       </c>
-      <c r="T819" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="820" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A820" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B820" s="4"/>
-      <c r="R820" t="s">
-        <v>307</v>
-      </c>
-      <c r="S820" s="4">
-        <f>-10.7/1000</f>
-        <v>-1.0699999999999999E-2</v>
-      </c>
       <c r="T820" t="s">
-        <v>310</v>
-      </c>
-      <c r="U820" t="s">
-        <v>321</v>
-      </c>
-      <c r="V820" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
     </row>
     <row r="821" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A821" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B821" s="4"/>
       <c r="R821" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="S821" s="4">
         <f>-10.7/1000</f>
         <v>-1.0699999999999999E-2</v>
       </c>
       <c r="T821" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="U821" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="V821" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="822" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="C822" t="s">
+      <c r="A822" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B822" s="4"/>
+      <c r="R822" t="s">
+        <v>306</v>
+      </c>
+      <c r="S822" s="4">
+        <f>-10.7/1000</f>
+        <v>-1.0699999999999999E-2</v>
+      </c>
+      <c r="T822" t="s">
+        <v>309</v>
+      </c>
+      <c r="U822" t="s">
+        <v>320</v>
+      </c>
+      <c r="V822" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="823" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="C823" t="s">
         <v>226</v>
       </c>
-      <c r="R822" t="s">
-        <v>307</v>
-      </c>
-      <c r="S822">
+      <c r="R823" t="s">
+        <v>306</v>
+      </c>
+      <c r="S823">
         <f>-0.6/1000</f>
         <v>-5.9999999999999995E-4</v>
       </c>
-      <c r="T822" t="s">
-        <v>310</v>
-      </c>
-      <c r="V822" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="823" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B823" t="s">
-        <v>337</v>
-      </c>
-      <c r="R823" t="s">
-        <v>307</v>
-      </c>
-      <c r="S823" s="29">
+      <c r="T823" t="s">
+        <v>309</v>
+      </c>
+      <c r="V823" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="824" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B824" t="s">
+        <v>336</v>
+      </c>
+      <c r="R824" t="s">
+        <v>306</v>
+      </c>
+      <c r="S824" s="29">
         <f>-20*0.45/0.85/1000</f>
         <v>-1.0588235294117647E-2</v>
       </c>
-      <c r="T823" t="s">
-        <v>310</v>
-      </c>
-      <c r="U823" t="s">
-        <v>339</v>
-      </c>
-      <c r="V823" t="s">
+      <c r="T824" t="s">
+        <v>309</v>
+      </c>
+      <c r="U824" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="825" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="D825" t="s">
-        <v>313</v>
-      </c>
-      <c r="R825" t="s">
-        <v>308</v>
-      </c>
-      <c r="S825">
+      <c r="V824" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="826" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="D826" t="s">
+        <v>312</v>
+      </c>
+      <c r="R826" t="s">
+        <v>307</v>
+      </c>
+      <c r="S826">
         <f>-9.2/1000</f>
         <v>-9.1999999999999998E-3</v>
       </c>
-      <c r="T825" t="s">
-        <v>310</v>
-      </c>
-      <c r="V825" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="827" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I827" t="s">
-        <v>107</v>
-      </c>
-      <c r="R827" t="s">
-        <v>316</v>
-      </c>
-      <c r="S827" s="31">
-        <v>-0.5</v>
-      </c>
-      <c r="T827" t="s">
-        <v>311</v>
-      </c>
-      <c r="V827" t="s">
-        <v>320</v>
+      <c r="T826" t="s">
+        <v>309</v>
+      </c>
+      <c r="V826" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="828" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I828" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R828" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="S828" s="31">
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="T828" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="V828" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="829" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I829" t="s">
+        <v>108</v>
+      </c>
+      <c r="R829" t="s">
+        <v>315</v>
+      </c>
+      <c r="S829" s="31">
+        <v>-1</v>
+      </c>
+      <c r="T829" t="s">
+        <v>310</v>
+      </c>
+      <c r="V829" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="830" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I830" t="s">
         <v>208</v>
       </c>
-      <c r="R829" t="s">
-        <v>316</v>
-      </c>
-      <c r="S829" s="22">
+      <c r="R830" t="s">
+        <v>315</v>
+      </c>
+      <c r="S830" s="22">
         <v>-1</v>
       </c>
-      <c r="T829" t="s">
-        <v>311</v>
-      </c>
-      <c r="U829" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="830" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R830" t="s">
-        <v>318</v>
-      </c>
-      <c r="S830" s="22">
-        <f>-0.4 / ( (2*30.97) / (2*30.97 + 5*16) )</f>
-        <v>-0.91662899580238943</v>
-      </c>
       <c r="T830" t="s">
-        <v>319</v>
-      </c>
-      <c r="U830" s="32" t="s">
-        <v>334</v>
-      </c>
-      <c r="V830" t="s">
-        <v>336</v>
+        <v>310</v>
+      </c>
+      <c r="U830" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="831" spans="1:22" x14ac:dyDescent="0.25">
@@ -14985,75 +14990,93 @@
         <v>317</v>
       </c>
       <c r="S831" s="22">
+        <f>-0.4 / ( (2*30.97) / (2*30.97 + 5*16) )</f>
+        <v>-0.91662899580238943</v>
+      </c>
+      <c r="T831" t="s">
+        <v>318</v>
+      </c>
+      <c r="U831" s="32" t="s">
+        <v>333</v>
+      </c>
+      <c r="V831" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="832" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R832" t="s">
+        <v>316</v>
+      </c>
+      <c r="S832" s="22">
         <f>0.6 / ( (2*39.1) / (2*39.1 + 16) )</f>
         <v>0.72276214833759589</v>
       </c>
-      <c r="T831" t="s">
-        <v>319</v>
-      </c>
-      <c r="U831" s="32" t="s">
+      <c r="T832" t="s">
+        <v>318</v>
+      </c>
+      <c r="U832" s="32" t="s">
+        <v>334</v>
+      </c>
+      <c r="V832" t="s">
         <v>335</v>
       </c>
-      <c r="V831" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="833" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="R833" t="s">
-        <v>309</v>
-      </c>
-      <c r="S833" s="31">
+    </row>
+    <row r="834" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="R834" t="s">
+        <v>308</v>
+      </c>
+      <c r="S834" s="31">
         <f>3/5</f>
         <v>0.6</v>
       </c>
-      <c r="T833" t="s">
-        <v>311</v>
-      </c>
-      <c r="U833" t="s">
-        <v>315</v>
-      </c>
-      <c r="V833" t="s">
+      <c r="T834" t="s">
+        <v>310</v>
+      </c>
+      <c r="U834" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="835" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="I835" t="s">
-        <v>326</v>
-      </c>
-      <c r="Q835" t="s">
-        <v>330</v>
-      </c>
-      <c r="R835" t="s">
-        <v>332</v>
-      </c>
-      <c r="S835" s="31">
+      <c r="V834" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="836" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="I836" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q836" t="s">
+        <v>329</v>
+      </c>
+      <c r="R836" t="s">
+        <v>331</v>
+      </c>
+      <c r="S836" s="31">
         <f>0.12*(44/12)</f>
         <v>0.43999999999999995</v>
       </c>
-      <c r="T835" t="s">
+      <c r="T836" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="837" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="I837" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q837" t="s">
+        <v>329</v>
+      </c>
+      <c r="R837" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="836" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="I836" t="s">
-        <v>340</v>
-      </c>
-      <c r="Q836" t="s">
-        <v>330</v>
-      </c>
-      <c r="R836" t="s">
-        <v>332</v>
-      </c>
-      <c r="S836" s="31">
+      <c r="S837" s="31">
         <f>0.13*(44/12)</f>
         <v>0.47666666666666668</v>
       </c>
-      <c r="T836" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="837" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="S837" s="11"/>
+      <c r="T837" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="838" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="S838" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Added factors for losses of CO2 and CH4 from organic soils + adjusted N2O-N factor for SNG
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2507" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2528" uniqueCount="360">
   <si>
     <t>f_crop</t>
   </si>
@@ -1080,10 +1080,25 @@
     <t>grass clover ley (avg. 20/40% clover) and three harvest</t>
   </si>
   <si>
-    <t>Not included in NIR, reported under forest</t>
-  </si>
-  <si>
-    <t>Pers. comm. Mattias Lindblad (2024-11-14)</t>
+    <t>kg/ha</t>
+  </si>
+  <si>
+    <t>kg CO2/ha</t>
+  </si>
+  <si>
+    <t>Not included in NIR under Agriculture, reported under forest</t>
+  </si>
+  <si>
+    <t>Lindgren &amp; Lundblad (2014) Towards new reporting of drained organic soils under the UNFCCC - assessment of emission factors and areas in Sweden.</t>
+  </si>
+  <si>
+    <t>Soil losses organic soils</t>
+  </si>
+  <si>
+    <t>CH4bio</t>
+  </si>
+  <si>
+    <t>kg CH4/ha</t>
   </si>
 </sst>
 </file>
@@ -1240,7 +1255,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1277,6 +1292,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1558,7 +1574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V838"/>
+  <dimension ref="A1:V845"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="21" customWidth="1"/>
@@ -14493,106 +14509,105 @@
       </c>
     </row>
     <row r="798" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="Q798" t="s">
+      <c r="A798" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="B798" s="2"/>
+      <c r="C798" s="2"/>
+      <c r="D798" s="2"/>
+      <c r="E798" s="2"/>
+      <c r="F798" s="2"/>
+      <c r="G798" s="2"/>
+      <c r="H798" s="2"/>
+      <c r="I798" s="2"/>
+      <c r="J798" s="2"/>
+      <c r="K798" s="2"/>
+      <c r="L798" s="2"/>
+      <c r="M798" s="2"/>
+      <c r="N798" s="2"/>
+      <c r="O798" s="2"/>
+      <c r="P798" s="2"/>
+      <c r="Q798" s="2"/>
+      <c r="R798" s="2"/>
+      <c r="S798" s="2"/>
+      <c r="T798" s="2"/>
+      <c r="U798" s="2"/>
+      <c r="V798" s="2"/>
+    </row>
+    <row r="799" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R799" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="S799" s="5">
+        <v>0</v>
+      </c>
+      <c r="T799" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="U799" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="801" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E801" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q801" t="s">
         <v>148</v>
       </c>
-      <c r="R798" t="s">
+      <c r="R801" t="s">
         <v>166</v>
       </c>
-      <c r="S798">
-        <v>0</v>
-      </c>
-      <c r="T798" t="s">
+      <c r="S801">
+        <v>13</v>
+      </c>
+      <c r="T801" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="799" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="E799" t="s">
+      <c r="V801" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="802" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E802" t="s">
         <v>175</v>
       </c>
-      <c r="Q799" t="s">
-        <v>148</v>
-      </c>
-      <c r="R799" t="s">
+      <c r="Q802" t="s">
+        <v>329</v>
+      </c>
+      <c r="R802" t="s">
         <v>166</v>
       </c>
-      <c r="S799">
-        <v>13</v>
-      </c>
-      <c r="T799" t="s">
-        <v>167</v>
-      </c>
-      <c r="V799" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="800" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="E800" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q800" t="s">
-        <v>148</v>
-      </c>
-      <c r="R800" t="s">
+      <c r="S802" s="34">
+        <f>6.1*(44/12)*1000</f>
+        <v>22366.666666666664</v>
+      </c>
+      <c r="T802" t="s">
+        <v>354</v>
+      </c>
+      <c r="V802" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="803" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E803" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q803" t="s">
+        <v>358</v>
+      </c>
+      <c r="R803" t="s">
         <v>166</v>
       </c>
-      <c r="S800">
-        <v>13</v>
-      </c>
-      <c r="T800" t="s">
-        <v>167</v>
-      </c>
-      <c r="U800" t="s">
-        <v>353</v>
-      </c>
-      <c r="V800" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="802" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A802" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B802" s="2"/>
-      <c r="C802" s="2"/>
-      <c r="D802" s="2"/>
-      <c r="E802" s="2"/>
-      <c r="F802" s="2"/>
-      <c r="G802" s="2"/>
-      <c r="H802" s="2"/>
-      <c r="I802" s="2"/>
-      <c r="J802" s="2"/>
-      <c r="K802" s="2"/>
-      <c r="L802" s="2"/>
-      <c r="M802" s="2"/>
-      <c r="N802" s="2"/>
-      <c r="O802" s="2"/>
-      <c r="P802" s="2"/>
-      <c r="Q802" s="2"/>
-      <c r="R802" s="2"/>
-      <c r="S802" s="2"/>
-      <c r="T802" s="2"/>
-      <c r="U802" s="2"/>
-      <c r="V802" s="2"/>
-    </row>
-    <row r="804" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="E804" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q804" t="s">
-        <v>173</v>
-      </c>
-      <c r="R804" t="s">
-        <v>170</v>
-      </c>
-      <c r="S804">
-        <v>0.24</v>
-      </c>
-      <c r="T804" t="s">
-        <v>172</v>
-      </c>
-      <c r="V804" t="s">
-        <v>171</v>
+      <c r="S803">
+        <f>0+58.3</f>
+        <v>58.3</v>
+      </c>
+      <c r="T803" t="s">
+        <v>359</v>
+      </c>
+      <c r="V803" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="805" spans="1:22" x14ac:dyDescent="0.25">
@@ -14600,483 +14615,594 @@
         <v>176</v>
       </c>
       <c r="Q805" t="s">
-        <v>173</v>
+        <v>148</v>
       </c>
       <c r="R805" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="S805">
-        <v>0.24</v>
+        <v>2.8</v>
       </c>
       <c r="T805" t="s">
-        <v>172</v>
+        <v>167</v>
+      </c>
+      <c r="U805" t="s">
+        <v>355</v>
       </c>
       <c r="V805" t="s">
-        <v>171</v>
+        <v>356</v>
       </c>
     </row>
     <row r="806" spans="1:22" x14ac:dyDescent="0.25">
       <c r="E806" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q806" t="s">
+        <v>329</v>
+      </c>
+      <c r="R806" t="s">
+        <v>166</v>
+      </c>
+      <c r="S806" s="34">
+        <f>2.6*(44/12)*1000</f>
+        <v>9533.3333333333339</v>
+      </c>
+      <c r="T806" t="s">
+        <v>354</v>
+      </c>
+      <c r="V806" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="807" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E807" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q807" t="s">
+        <v>358</v>
+      </c>
+      <c r="R807" t="s">
+        <v>166</v>
+      </c>
+      <c r="S807">
+        <f>2.5+5.4</f>
+        <v>7.9</v>
+      </c>
+      <c r="T807" t="s">
+        <v>359</v>
+      </c>
+      <c r="V807" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="809" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A809" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B809" s="2"/>
+      <c r="C809" s="2"/>
+      <c r="D809" s="2"/>
+      <c r="E809" s="2"/>
+      <c r="F809" s="2"/>
+      <c r="G809" s="2"/>
+      <c r="H809" s="2"/>
+      <c r="I809" s="2"/>
+      <c r="J809" s="2"/>
+      <c r="K809" s="2"/>
+      <c r="L809" s="2"/>
+      <c r="M809" s="2"/>
+      <c r="N809" s="2"/>
+      <c r="O809" s="2"/>
+      <c r="P809" s="2"/>
+      <c r="Q809" s="2"/>
+      <c r="R809" s="2"/>
+      <c r="S809" s="2"/>
+      <c r="T809" s="2"/>
+      <c r="U809" s="2"/>
+      <c r="V809" s="2"/>
+    </row>
+    <row r="811" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E811" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q811" t="s">
+        <v>173</v>
+      </c>
+      <c r="R811" t="s">
+        <v>170</v>
+      </c>
+      <c r="S811">
+        <v>0.24</v>
+      </c>
+      <c r="T811" t="s">
+        <v>172</v>
+      </c>
+      <c r="V811" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="812" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E812" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q812" t="s">
+        <v>173</v>
+      </c>
+      <c r="R812" t="s">
+        <v>170</v>
+      </c>
+      <c r="S812">
+        <v>0.24</v>
+      </c>
+      <c r="T812" t="s">
+        <v>172</v>
+      </c>
+      <c r="V812" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="813" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E813" t="s">
         <v>177</v>
       </c>
-      <c r="Q806" t="s">
+      <c r="Q813" t="s">
         <v>173</v>
       </c>
-      <c r="R806" t="s">
+      <c r="R813" t="s">
         <v>170</v>
       </c>
-      <c r="S806">
+      <c r="S813">
         <v>0</v>
       </c>
-      <c r="T806" t="s">
+      <c r="T813" t="s">
         <v>172</v>
       </c>
-      <c r="U806" t="s">
+      <c r="U813" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="808" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A808" s="27" t="s">
+    <row r="815" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A815" s="27" t="s">
         <v>305</v>
       </c>
-      <c r="B808" s="27"/>
-      <c r="C808" s="28"/>
-      <c r="D808" s="28"/>
-      <c r="E808" s="28"/>
-      <c r="F808" s="28"/>
-      <c r="G808" s="28"/>
-      <c r="H808" s="28"/>
-      <c r="I808" s="28"/>
-      <c r="J808" s="28"/>
-      <c r="K808" s="28"/>
-      <c r="L808" s="28"/>
-      <c r="M808" s="28"/>
-      <c r="N808" s="28"/>
-      <c r="O808" s="28"/>
-      <c r="P808" s="28"/>
-      <c r="Q808" s="28"/>
-      <c r="R808" s="28"/>
-      <c r="S808" s="28"/>
-      <c r="T808" s="28"/>
-      <c r="U808" s="28"/>
-      <c r="V808" s="28"/>
-    </row>
-    <row r="810" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I810" t="s">
+      <c r="B815" s="27"/>
+      <c r="C815" s="28"/>
+      <c r="D815" s="28"/>
+      <c r="E815" s="28"/>
+      <c r="F815" s="28"/>
+      <c r="G815" s="28"/>
+      <c r="H815" s="28"/>
+      <c r="I815" s="28"/>
+      <c r="J815" s="28"/>
+      <c r="K815" s="28"/>
+      <c r="L815" s="28"/>
+      <c r="M815" s="28"/>
+      <c r="N815" s="28"/>
+      <c r="O815" s="28"/>
+      <c r="P815" s="28"/>
+      <c r="Q815" s="28"/>
+      <c r="R815" s="28"/>
+      <c r="S815" s="28"/>
+      <c r="T815" s="28"/>
+      <c r="U815" s="28"/>
+      <c r="V815" s="28"/>
+    </row>
+    <row r="817" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I817" t="s">
         <v>325</v>
       </c>
-      <c r="R810" t="s">
+      <c r="R817" t="s">
         <v>323</v>
       </c>
-      <c r="S810" s="11">
+      <c r="S817" s="11">
         <f>213/(213 + 60)*100</f>
         <v>78.021978021978029</v>
       </c>
-      <c r="T810" t="s">
+      <c r="T817" t="s">
         <v>97</v>
       </c>
-      <c r="V810" t="s">
+      <c r="V817" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="811" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I811" t="s">
+    <row r="818" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I818" t="s">
         <v>339</v>
       </c>
-      <c r="R811" t="s">
+      <c r="R818" t="s">
         <v>323</v>
       </c>
-      <c r="S811" s="11">
+      <c r="S818" s="11">
         <f>60/(213 + 60)*100</f>
         <v>21.978021978021978</v>
       </c>
-      <c r="T811" t="s">
+      <c r="T818" t="s">
         <v>97</v>
       </c>
-      <c r="V811" t="s">
+      <c r="V818" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="813" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I813" t="s">
+    <row r="820" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I820" t="s">
         <v>325</v>
       </c>
-      <c r="R813" t="s">
+      <c r="R820" t="s">
         <v>326</v>
       </c>
-      <c r="S813">
+      <c r="S820">
         <v>45</v>
       </c>
-      <c r="T813" t="s">
+      <c r="T820" t="s">
         <v>97</v>
       </c>
-      <c r="V813" t="s">
+      <c r="V820" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="814" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I814" t="s">
+    <row r="821" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I821" t="s">
         <v>339</v>
       </c>
-      <c r="R814" t="s">
+      <c r="R821" t="s">
         <v>326</v>
       </c>
-      <c r="S814">
+      <c r="S821">
         <v>48</v>
       </c>
-      <c r="T814" t="s">
+      <c r="T821" t="s">
         <v>97</v>
       </c>
-      <c r="V814" t="s">
+      <c r="V821" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="816" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R816" t="s">
+    <row r="823" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R823" t="s">
         <v>306</v>
       </c>
-      <c r="S816" s="30">
-        <f>S823</f>
+      <c r="S823" s="30">
+        <f>S830</f>
         <v>-5.9999999999999995E-4</v>
       </c>
-      <c r="T816" t="s">
+      <c r="T823" t="s">
         <v>309</v>
       </c>
-      <c r="U816" t="s">
+      <c r="U823" t="s">
         <v>322</v>
       </c>
-      <c r="V816" t="s">
+      <c r="V823" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="817" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A817" t="s">
+    <row r="824" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A824" t="s">
         <v>37</v>
       </c>
-      <c r="G817" t="s">
+      <c r="G824" t="s">
         <v>142</v>
       </c>
-      <c r="R817" t="s">
+      <c r="R824" t="s">
         <v>306</v>
       </c>
-      <c r="S817" s="29">
+      <c r="S824" s="29">
         <f>-(45.5*0.1+10.7*0.9)/1000</f>
         <v>-1.418E-2</v>
       </c>
-      <c r="T817" t="s">
+      <c r="T824" t="s">
         <v>309</v>
       </c>
-      <c r="U817" t="s">
+      <c r="U824" t="s">
         <v>340</v>
       </c>
-      <c r="V817" t="s">
+      <c r="V824" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="818" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A818" t="s">
+    <row r="825" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A825" t="s">
         <v>38</v>
       </c>
-      <c r="G818" t="s">
+      <c r="G825" t="s">
         <v>142</v>
       </c>
-      <c r="R818" t="s">
+      <c r="R825" t="s">
         <v>306</v>
       </c>
-      <c r="S818" s="33">
-        <f>S817</f>
+      <c r="S825" s="33">
+        <f>S824</f>
         <v>-1.418E-2</v>
       </c>
-      <c r="T818" t="s">
+      <c r="T825" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="819" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A819" t="s">
+    <row r="826" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A826" t="s">
         <v>37</v>
       </c>
-      <c r="G819" t="s">
+      <c r="G826" t="s">
         <v>98</v>
       </c>
-      <c r="R819" t="s">
+      <c r="R826" t="s">
         <v>306</v>
       </c>
-      <c r="S819" s="29">
+      <c r="S826" s="29">
         <f>-(45.5*0.4+10.7*0.6)/1000</f>
         <v>-2.4619999999999996E-2</v>
       </c>
-      <c r="T819" t="s">
+      <c r="T826" t="s">
         <v>309</v>
       </c>
-      <c r="U819" t="s">
+      <c r="U826" t="s">
         <v>341</v>
       </c>
-      <c r="V819" t="s">
+      <c r="V826" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="820" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A820" t="s">
+    <row r="827" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A827" t="s">
         <v>38</v>
       </c>
-      <c r="G820" t="s">
+      <c r="G827" t="s">
         <v>98</v>
       </c>
-      <c r="R820" t="s">
+      <c r="R827" t="s">
         <v>306</v>
       </c>
-      <c r="S820" s="33">
-        <f>S819</f>
+      <c r="S827" s="33">
+        <f>S826</f>
         <v>-2.4619999999999996E-2</v>
       </c>
-      <c r="T820" t="s">
+      <c r="T827" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="821" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A821" s="4" t="s">
+    <row r="828" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A828" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B821" s="4"/>
-      <c r="R821" t="s">
+      <c r="B828" s="4"/>
+      <c r="R828" t="s">
         <v>306</v>
       </c>
-      <c r="S821" s="4">
+      <c r="S828" s="4">
         <f>-10.7/1000</f>
         <v>-1.0699999999999999E-2</v>
       </c>
-      <c r="T821" t="s">
+      <c r="T828" t="s">
         <v>309</v>
       </c>
-      <c r="U821" t="s">
+      <c r="U828" t="s">
         <v>320</v>
       </c>
-      <c r="V821" t="s">
+      <c r="V828" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="822" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A822" s="4" t="s">
+    <row r="829" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A829" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B822" s="4"/>
-      <c r="R822" t="s">
+      <c r="B829" s="4"/>
+      <c r="R829" t="s">
         <v>306</v>
       </c>
-      <c r="S822" s="4">
+      <c r="S829" s="4">
         <f>-10.7/1000</f>
         <v>-1.0699999999999999E-2</v>
       </c>
-      <c r="T822" t="s">
+      <c r="T829" t="s">
         <v>309</v>
       </c>
-      <c r="U822" t="s">
+      <c r="U829" t="s">
         <v>320</v>
       </c>
-      <c r="V822" t="s">
+      <c r="V829" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="823" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="C823" t="s">
+    <row r="830" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="C830" t="s">
         <v>226</v>
       </c>
-      <c r="R823" t="s">
+      <c r="R830" t="s">
         <v>306</v>
       </c>
-      <c r="S823">
+      <c r="S830">
         <f>-0.6/1000</f>
         <v>-5.9999999999999995E-4</v>
       </c>
-      <c r="T823" t="s">
+      <c r="T830" t="s">
         <v>309</v>
       </c>
-      <c r="V823" t="s">
+      <c r="V830" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="824" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B824" t="s">
+    <row r="831" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B831" t="s">
         <v>336</v>
       </c>
-      <c r="R824" t="s">
+      <c r="R831" t="s">
         <v>306</v>
       </c>
-      <c r="S824" s="29">
+      <c r="S831" s="29">
         <f>-20*0.45/0.85/1000</f>
         <v>-1.0588235294117647E-2</v>
       </c>
-      <c r="T824" t="s">
+      <c r="T831" t="s">
         <v>309</v>
       </c>
-      <c r="U824" t="s">
+      <c r="U831" t="s">
         <v>338</v>
       </c>
-      <c r="V824" t="s">
+      <c r="V831" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="826" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="D826" t="s">
+    <row r="833" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="D833" t="s">
         <v>312</v>
       </c>
-      <c r="R826" t="s">
+      <c r="R833" t="s">
         <v>307</v>
       </c>
-      <c r="S826">
+      <c r="S833">
         <f>-9.2/1000</f>
         <v>-9.1999999999999998E-3</v>
       </c>
-      <c r="T826" t="s">
+      <c r="T833" t="s">
         <v>309</v>
       </c>
-      <c r="V826" t="s">
+      <c r="V833" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="828" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I828" t="s">
+    <row r="835" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I835" t="s">
         <v>107</v>
       </c>
-      <c r="R828" t="s">
+      <c r="R835" t="s">
         <v>315</v>
       </c>
-      <c r="S828" s="31">
+      <c r="S835" s="31">
         <v>-0.5</v>
       </c>
-      <c r="T828" t="s">
+      <c r="T835" t="s">
         <v>310</v>
       </c>
-      <c r="V828" t="s">
+      <c r="V835" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="829" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I829" t="s">
+    <row r="836" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I836" t="s">
         <v>108</v>
       </c>
-      <c r="R829" t="s">
+      <c r="R836" t="s">
         <v>315</v>
       </c>
-      <c r="S829" s="31">
+      <c r="S836" s="31">
         <v>-1</v>
       </c>
-      <c r="T829" t="s">
+      <c r="T836" t="s">
         <v>310</v>
       </c>
-      <c r="V829" t="s">
+      <c r="V836" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="830" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I830" t="s">
+    <row r="837" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I837" t="s">
         <v>208</v>
       </c>
-      <c r="R830" t="s">
+      <c r="R837" t="s">
         <v>315</v>
       </c>
-      <c r="S830" s="22">
+      <c r="S837" s="22">
         <v>-1</v>
       </c>
-      <c r="T830" t="s">
+      <c r="T837" t="s">
         <v>310</v>
       </c>
-      <c r="U830" t="s">
+      <c r="U837" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="831" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R831" t="s">
+    <row r="838" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="R838" t="s">
         <v>317</v>
       </c>
-      <c r="S831" s="22">
+      <c r="S838" s="22">
         <f>-0.4 / ( (2*30.97) / (2*30.97 + 5*16) )</f>
         <v>-0.91662899580238943</v>
       </c>
-      <c r="T831" t="s">
+      <c r="T838" t="s">
         <v>318</v>
       </c>
-      <c r="U831" s="32" t="s">
+      <c r="U838" s="32" t="s">
         <v>333</v>
       </c>
-      <c r="V831" t="s">
+      <c r="V838" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="832" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R832" t="s">
+    <row r="839" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="R839" t="s">
         <v>316</v>
       </c>
-      <c r="S832" s="22">
+      <c r="S839" s="22">
         <f>0.6 / ( (2*39.1) / (2*39.1 + 16) )</f>
         <v>0.72276214833759589</v>
       </c>
-      <c r="T832" t="s">
+      <c r="T839" t="s">
         <v>318</v>
       </c>
-      <c r="U832" s="32" t="s">
+      <c r="U839" s="32" t="s">
         <v>334</v>
       </c>
-      <c r="V832" t="s">
+      <c r="V839" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="834" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="R834" t="s">
+    <row r="841" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="R841" t="s">
         <v>308</v>
       </c>
-      <c r="S834" s="31">
+      <c r="S841" s="31">
         <f>3/5</f>
         <v>0.6</v>
       </c>
-      <c r="T834" t="s">
+      <c r="T841" t="s">
         <v>310</v>
       </c>
-      <c r="U834" t="s">
+      <c r="U841" t="s">
         <v>314</v>
       </c>
-      <c r="V834" t="s">
+      <c r="V841" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="836" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="I836" t="s">
+    <row r="843" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I843" t="s">
         <v>325</v>
       </c>
-      <c r="Q836" t="s">
+      <c r="Q843" t="s">
         <v>329</v>
       </c>
-      <c r="R836" t="s">
+      <c r="R843" t="s">
         <v>331</v>
       </c>
-      <c r="S836" s="31">
+      <c r="S843" s="31">
         <f>0.12*(44/12)</f>
         <v>0.43999999999999995</v>
       </c>
-      <c r="T836" t="s">
+      <c r="T843" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="837" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="I837" t="s">
+    <row r="844" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I844" t="s">
         <v>339</v>
       </c>
-      <c r="Q837" t="s">
+      <c r="Q844" t="s">
         <v>329</v>
       </c>
-      <c r="R837" t="s">
+      <c r="R844" t="s">
         <v>331</v>
       </c>
-      <c r="S837" s="31">
+      <c r="S844" s="31">
         <f>0.13*(44/12)</f>
         <v>0.47666666666666668</v>
       </c>
-      <c r="T837" t="s">
+      <c r="T844" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="838" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="S838" s="11"/>
+    <row r="845" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="S845" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Added EF for N2O-N from N in cover crop residues
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2528" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2532" uniqueCount="362">
   <si>
     <t>f_crop</t>
   </si>
@@ -1099,6 +1099,12 @@
   </si>
   <si>
     <t>kg CH4/ha</t>
+  </si>
+  <si>
+    <t>soil_losses_cover_crop_residues</t>
+  </si>
+  <si>
+    <t>cover crop residues</t>
   </si>
 </sst>
 </file>
@@ -1110,7 +1116,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1215,6 +1221,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-9.9978637043366805E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1255,7 +1268,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1293,6 +1306,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1574,7 +1588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V845"/>
+  <dimension ref="A1:V846"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="21" customWidth="1"/>
@@ -14508,64 +14522,62 @@
         <v>151</v>
       </c>
     </row>
-    <row r="798" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A798" s="2" t="s">
+    <row r="797" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="Q797" t="s">
+        <v>148</v>
+      </c>
+      <c r="R797" t="s">
+        <v>360</v>
+      </c>
+      <c r="S797" s="35">
+        <f>S796</f>
+        <v>1</v>
+      </c>
+      <c r="T797" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="U797" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="799" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A799" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="B798" s="2"/>
-      <c r="C798" s="2"/>
-      <c r="D798" s="2"/>
-      <c r="E798" s="2"/>
-      <c r="F798" s="2"/>
-      <c r="G798" s="2"/>
-      <c r="H798" s="2"/>
-      <c r="I798" s="2"/>
-      <c r="J798" s="2"/>
-      <c r="K798" s="2"/>
-      <c r="L798" s="2"/>
-      <c r="M798" s="2"/>
-      <c r="N798" s="2"/>
-      <c r="O798" s="2"/>
-      <c r="P798" s="2"/>
-      <c r="Q798" s="2"/>
-      <c r="R798" s="2"/>
-      <c r="S798" s="2"/>
-      <c r="T798" s="2"/>
-      <c r="U798" s="2"/>
-      <c r="V798" s="2"/>
-    </row>
-    <row r="799" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R799" s="5" t="s">
+      <c r="B799" s="2"/>
+      <c r="C799" s="2"/>
+      <c r="D799" s="2"/>
+      <c r="E799" s="2"/>
+      <c r="F799" s="2"/>
+      <c r="G799" s="2"/>
+      <c r="H799" s="2"/>
+      <c r="I799" s="2"/>
+      <c r="J799" s="2"/>
+      <c r="K799" s="2"/>
+      <c r="L799" s="2"/>
+      <c r="M799" s="2"/>
+      <c r="N799" s="2"/>
+      <c r="O799" s="2"/>
+      <c r="P799" s="2"/>
+      <c r="Q799" s="2"/>
+      <c r="R799" s="2"/>
+      <c r="S799" s="2"/>
+      <c r="T799" s="2"/>
+      <c r="U799" s="2"/>
+      <c r="V799" s="2"/>
+    </row>
+    <row r="800" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R800" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="S799" s="5">
+      <c r="S800" s="5">
         <v>0</v>
       </c>
-      <c r="T799" s="5" t="s">
+      <c r="T800" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="U799" s="5" t="s">
+      <c r="U800" s="5" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="801" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="E801" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q801" t="s">
-        <v>148</v>
-      </c>
-      <c r="R801" t="s">
-        <v>166</v>
-      </c>
-      <c r="S801">
-        <v>13</v>
-      </c>
-      <c r="T801" t="s">
-        <v>167</v>
-      </c>
-      <c r="V801" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="802" spans="1:22" x14ac:dyDescent="0.25">
@@ -14573,20 +14585,19 @@
         <v>175</v>
       </c>
       <c r="Q802" t="s">
-        <v>329</v>
+        <v>148</v>
       </c>
       <c r="R802" t="s">
         <v>166</v>
       </c>
-      <c r="S802" s="34">
-        <f>6.1*(44/12)*1000</f>
-        <v>22366.666666666664</v>
+      <c r="S802">
+        <v>13</v>
       </c>
       <c r="T802" t="s">
-        <v>354</v>
+        <v>167</v>
       </c>
       <c r="V802" t="s">
-        <v>356</v>
+        <v>151</v>
       </c>
     </row>
     <row r="803" spans="1:22" x14ac:dyDescent="0.25">
@@ -14594,42 +14605,40 @@
         <v>175</v>
       </c>
       <c r="Q803" t="s">
-        <v>358</v>
+        <v>329</v>
       </c>
       <c r="R803" t="s">
         <v>166</v>
       </c>
-      <c r="S803">
+      <c r="S803" s="34">
+        <f>6.1*(44/12)*1000</f>
+        <v>22366.666666666664</v>
+      </c>
+      <c r="T803" t="s">
+        <v>354</v>
+      </c>
+      <c r="V803" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="804" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E804" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q804" t="s">
+        <v>358</v>
+      </c>
+      <c r="R804" t="s">
+        <v>166</v>
+      </c>
+      <c r="S804">
         <f>0+58.3</f>
         <v>58.3</v>
       </c>
-      <c r="T803" t="s">
+      <c r="T804" t="s">
         <v>359</v>
       </c>
-      <c r="V803" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="805" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="E805" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q805" t="s">
-        <v>148</v>
-      </c>
-      <c r="R805" t="s">
-        <v>166</v>
-      </c>
-      <c r="S805">
-        <v>2.8</v>
-      </c>
-      <c r="T805" t="s">
-        <v>167</v>
-      </c>
-      <c r="U805" t="s">
-        <v>355</v>
-      </c>
-      <c r="V805" t="s">
+      <c r="V804" t="s">
         <v>356</v>
       </c>
     </row>
@@ -14638,17 +14647,19 @@
         <v>176</v>
       </c>
       <c r="Q806" t="s">
-        <v>329</v>
+        <v>148</v>
       </c>
       <c r="R806" t="s">
         <v>166</v>
       </c>
-      <c r="S806" s="34">
-        <f>2.6*(44/12)*1000</f>
-        <v>9533.3333333333339</v>
+      <c r="S806">
+        <v>2.8</v>
       </c>
       <c r="T806" t="s">
-        <v>354</v>
+        <v>167</v>
+      </c>
+      <c r="U806" t="s">
+        <v>355</v>
       </c>
       <c r="V806" t="s">
         <v>356</v>
@@ -14659,71 +14670,72 @@
         <v>176</v>
       </c>
       <c r="Q807" t="s">
-        <v>358</v>
+        <v>329</v>
       </c>
       <c r="R807" t="s">
         <v>166</v>
       </c>
-      <c r="S807">
+      <c r="S807" s="34">
+        <f>2.6*(44/12)*1000</f>
+        <v>9533.3333333333339</v>
+      </c>
+      <c r="T807" t="s">
+        <v>354</v>
+      </c>
+      <c r="V807" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="808" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E808" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q808" t="s">
+        <v>358</v>
+      </c>
+      <c r="R808" t="s">
+        <v>166</v>
+      </c>
+      <c r="S808">
         <f>2.5+5.4</f>
         <v>7.9</v>
       </c>
-      <c r="T807" t="s">
+      <c r="T808" t="s">
         <v>359</v>
       </c>
-      <c r="V807" t="s">
+      <c r="V808" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="809" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A809" s="2" t="s">
+    <row r="810" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A810" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B809" s="2"/>
-      <c r="C809" s="2"/>
-      <c r="D809" s="2"/>
-      <c r="E809" s="2"/>
-      <c r="F809" s="2"/>
-      <c r="G809" s="2"/>
-      <c r="H809" s="2"/>
-      <c r="I809" s="2"/>
-      <c r="J809" s="2"/>
-      <c r="K809" s="2"/>
-      <c r="L809" s="2"/>
-      <c r="M809" s="2"/>
-      <c r="N809" s="2"/>
-      <c r="O809" s="2"/>
-      <c r="P809" s="2"/>
-      <c r="Q809" s="2"/>
-      <c r="R809" s="2"/>
-      <c r="S809" s="2"/>
-      <c r="T809" s="2"/>
-      <c r="U809" s="2"/>
-      <c r="V809" s="2"/>
-    </row>
-    <row r="811" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="E811" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q811" t="s">
-        <v>173</v>
-      </c>
-      <c r="R811" t="s">
-        <v>170</v>
-      </c>
-      <c r="S811">
-        <v>0.24</v>
-      </c>
-      <c r="T811" t="s">
-        <v>172</v>
-      </c>
-      <c r="V811" t="s">
-        <v>171</v>
-      </c>
+      <c r="B810" s="2"/>
+      <c r="C810" s="2"/>
+      <c r="D810" s="2"/>
+      <c r="E810" s="2"/>
+      <c r="F810" s="2"/>
+      <c r="G810" s="2"/>
+      <c r="H810" s="2"/>
+      <c r="I810" s="2"/>
+      <c r="J810" s="2"/>
+      <c r="K810" s="2"/>
+      <c r="L810" s="2"/>
+      <c r="M810" s="2"/>
+      <c r="N810" s="2"/>
+      <c r="O810" s="2"/>
+      <c r="P810" s="2"/>
+      <c r="Q810" s="2"/>
+      <c r="R810" s="2"/>
+      <c r="S810" s="2"/>
+      <c r="T810" s="2"/>
+      <c r="U810" s="2"/>
+      <c r="V810" s="2"/>
     </row>
     <row r="812" spans="1:22" x14ac:dyDescent="0.25">
       <c r="E812" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q812" t="s">
         <v>173</v>
@@ -14743,7 +14755,7 @@
     </row>
     <row r="813" spans="1:22" x14ac:dyDescent="0.25">
       <c r="E813" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q813" t="s">
         <v>173</v>
@@ -14752,103 +14764,106 @@
         <v>170</v>
       </c>
       <c r="S813">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="T813" t="s">
         <v>172</v>
       </c>
-      <c r="U813" t="s">
+      <c r="V813" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="814" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E814" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q814" t="s">
+        <v>173</v>
+      </c>
+      <c r="R814" t="s">
+        <v>170</v>
+      </c>
+      <c r="S814">
+        <v>0</v>
+      </c>
+      <c r="T814" t="s">
+        <v>172</v>
+      </c>
+      <c r="U814" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="815" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A815" s="27" t="s">
+    <row r="816" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A816" s="27" t="s">
         <v>305</v>
       </c>
-      <c r="B815" s="27"/>
-      <c r="C815" s="28"/>
-      <c r="D815" s="28"/>
-      <c r="E815" s="28"/>
-      <c r="F815" s="28"/>
-      <c r="G815" s="28"/>
-      <c r="H815" s="28"/>
-      <c r="I815" s="28"/>
-      <c r="J815" s="28"/>
-      <c r="K815" s="28"/>
-      <c r="L815" s="28"/>
-      <c r="M815" s="28"/>
-      <c r="N815" s="28"/>
-      <c r="O815" s="28"/>
-      <c r="P815" s="28"/>
-      <c r="Q815" s="28"/>
-      <c r="R815" s="28"/>
-      <c r="S815" s="28"/>
-      <c r="T815" s="28"/>
-      <c r="U815" s="28"/>
-      <c r="V815" s="28"/>
-    </row>
-    <row r="817" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I817" t="s">
+      <c r="B816" s="27"/>
+      <c r="C816" s="28"/>
+      <c r="D816" s="28"/>
+      <c r="E816" s="28"/>
+      <c r="F816" s="28"/>
+      <c r="G816" s="28"/>
+      <c r="H816" s="28"/>
+      <c r="I816" s="28"/>
+      <c r="J816" s="28"/>
+      <c r="K816" s="28"/>
+      <c r="L816" s="28"/>
+      <c r="M816" s="28"/>
+      <c r="N816" s="28"/>
+      <c r="O816" s="28"/>
+      <c r="P816" s="28"/>
+      <c r="Q816" s="28"/>
+      <c r="R816" s="28"/>
+      <c r="S816" s="28"/>
+      <c r="T816" s="28"/>
+      <c r="U816" s="28"/>
+      <c r="V816" s="28"/>
+    </row>
+    <row r="818" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I818" t="s">
         <v>325</v>
       </c>
-      <c r="R817" t="s">
+      <c r="R818" t="s">
         <v>323</v>
       </c>
-      <c r="S817" s="11">
+      <c r="S818" s="11">
         <f>213/(213 + 60)*100</f>
         <v>78.021978021978029</v>
       </c>
-      <c r="T817" t="s">
+      <c r="T818" t="s">
         <v>97</v>
       </c>
-      <c r="V817" t="s">
+      <c r="V818" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="818" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I818" t="s">
+    <row r="819" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I819" t="s">
         <v>339</v>
       </c>
-      <c r="R818" t="s">
+      <c r="R819" t="s">
         <v>323</v>
       </c>
-      <c r="S818" s="11">
+      <c r="S819" s="11">
         <f>60/(213 + 60)*100</f>
         <v>21.978021978021978</v>
       </c>
-      <c r="T818" t="s">
+      <c r="T819" t="s">
         <v>97</v>
       </c>
-      <c r="V818" t="s">
+      <c r="V819" t="s">
         <v>324</v>
-      </c>
-    </row>
-    <row r="820" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I820" t="s">
-        <v>325</v>
-      </c>
-      <c r="R820" t="s">
-        <v>326</v>
-      </c>
-      <c r="S820">
-        <v>45</v>
-      </c>
-      <c r="T820" t="s">
-        <v>97</v>
-      </c>
-      <c r="V820" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="821" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I821" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="R821" t="s">
         <v>326</v>
       </c>
       <c r="S821">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="T821" t="s">
         <v>97</v>
@@ -14857,133 +14872,128 @@
         <v>327</v>
       </c>
     </row>
-    <row r="823" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R823" t="s">
-        <v>306</v>
-      </c>
-      <c r="S823" s="30">
-        <f>S830</f>
-        <v>-5.9999999999999995E-4</v>
-      </c>
-      <c r="T823" t="s">
-        <v>309</v>
-      </c>
-      <c r="U823" t="s">
-        <v>322</v>
-      </c>
-      <c r="V823" t="s">
-        <v>313</v>
+    <row r="822" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="I822" t="s">
+        <v>339</v>
+      </c>
+      <c r="R822" t="s">
+        <v>326</v>
+      </c>
+      <c r="S822">
+        <v>48</v>
+      </c>
+      <c r="T822" t="s">
+        <v>97</v>
+      </c>
+      <c r="V822" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="824" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A824" t="s">
-        <v>37</v>
-      </c>
-      <c r="G824" t="s">
-        <v>142</v>
-      </c>
       <c r="R824" t="s">
         <v>306</v>
       </c>
-      <c r="S824" s="29">
+      <c r="S824" s="30">
+        <f>S831</f>
+        <v>-5.9999999999999995E-4</v>
+      </c>
+      <c r="T824" t="s">
+        <v>309</v>
+      </c>
+      <c r="U824" t="s">
+        <v>322</v>
+      </c>
+      <c r="V824" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="825" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A825" t="s">
+        <v>37</v>
+      </c>
+      <c r="G825" t="s">
+        <v>142</v>
+      </c>
+      <c r="R825" t="s">
+        <v>306</v>
+      </c>
+      <c r="S825" s="29">
         <f>-(45.5*0.1+10.7*0.9)/1000</f>
         <v>-1.418E-2</v>
       </c>
-      <c r="T824" t="s">
-        <v>309</v>
-      </c>
-      <c r="U824" t="s">
-        <v>340</v>
-      </c>
-      <c r="V824" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="825" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A825" t="s">
-        <v>38</v>
-      </c>
-      <c r="G825" t="s">
-        <v>142</v>
-      </c>
-      <c r="R825" t="s">
-        <v>306</v>
-      </c>
-      <c r="S825" s="33">
-        <f>S824</f>
-        <v>-1.418E-2</v>
-      </c>
       <c r="T825" t="s">
         <v>309</v>
       </c>
+      <c r="U825" t="s">
+        <v>340</v>
+      </c>
+      <c r="V825" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="826" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A826" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G826" t="s">
-        <v>98</v>
+        <v>142</v>
       </c>
       <c r="R826" t="s">
         <v>306</v>
       </c>
-      <c r="S826" s="29">
+      <c r="S826" s="33">
+        <f>S825</f>
+        <v>-1.418E-2</v>
+      </c>
+      <c r="T826" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="827" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A827" t="s">
+        <v>37</v>
+      </c>
+      <c r="G827" t="s">
+        <v>98</v>
+      </c>
+      <c r="R827" t="s">
+        <v>306</v>
+      </c>
+      <c r="S827" s="29">
         <f>-(45.5*0.4+10.7*0.6)/1000</f>
         <v>-2.4619999999999996E-2</v>
       </c>
-      <c r="T826" t="s">
-        <v>309</v>
-      </c>
-      <c r="U826" t="s">
-        <v>341</v>
-      </c>
-      <c r="V826" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="827" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A827" t="s">
-        <v>38</v>
-      </c>
-      <c r="G827" t="s">
-        <v>98</v>
-      </c>
-      <c r="R827" t="s">
-        <v>306</v>
-      </c>
-      <c r="S827" s="33">
-        <f>S826</f>
-        <v>-2.4619999999999996E-2</v>
-      </c>
       <c r="T827" t="s">
         <v>309</v>
       </c>
+      <c r="U827" t="s">
+        <v>341</v>
+      </c>
+      <c r="V827" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="828" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A828" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B828" s="4"/>
+      <c r="A828" t="s">
+        <v>38</v>
+      </c>
+      <c r="G828" t="s">
+        <v>98</v>
+      </c>
       <c r="R828" t="s">
         <v>306</v>
       </c>
-      <c r="S828" s="4">
-        <f>-10.7/1000</f>
-        <v>-1.0699999999999999E-2</v>
+      <c r="S828" s="33">
+        <f>S827</f>
+        <v>-2.4619999999999996E-2</v>
       </c>
       <c r="T828" t="s">
         <v>309</v>
       </c>
-      <c r="U828" t="s">
-        <v>320</v>
-      </c>
-      <c r="V828" t="s">
-        <v>313</v>
-      </c>
     </row>
     <row r="829" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A829" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B829" s="4"/>
       <c r="R829" t="s">
@@ -15004,88 +15014,93 @@
       </c>
     </row>
     <row r="830" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="C830" t="s">
-        <v>226</v>
-      </c>
+      <c r="A830" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B830" s="4"/>
       <c r="R830" t="s">
         <v>306</v>
       </c>
-      <c r="S830">
+      <c r="S830" s="4">
+        <f>-10.7/1000</f>
+        <v>-1.0699999999999999E-2</v>
+      </c>
+      <c r="T830" t="s">
+        <v>309</v>
+      </c>
+      <c r="U830" t="s">
+        <v>320</v>
+      </c>
+      <c r="V830" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="831" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="C831" t="s">
+        <v>226</v>
+      </c>
+      <c r="R831" t="s">
+        <v>306</v>
+      </c>
+      <c r="S831">
         <f>-0.6/1000</f>
         <v>-5.9999999999999995E-4</v>
       </c>
-      <c r="T830" t="s">
+      <c r="T831" t="s">
         <v>309</v>
       </c>
-      <c r="V830" t="s">
+      <c r="V831" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="831" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B831" t="s">
+    <row r="832" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B832" t="s">
         <v>336</v>
       </c>
-      <c r="R831" t="s">
+      <c r="R832" t="s">
         <v>306</v>
       </c>
-      <c r="S831" s="29">
+      <c r="S832" s="29">
         <f>-20*0.45/0.85/1000</f>
         <v>-1.0588235294117647E-2</v>
       </c>
-      <c r="T831" t="s">
+      <c r="T832" t="s">
         <v>309</v>
       </c>
-      <c r="U831" t="s">
+      <c r="U832" t="s">
         <v>338</v>
       </c>
-      <c r="V831" t="s">
+      <c r="V832" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="833" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="D833" t="s">
+    <row r="834" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="D834" t="s">
         <v>312</v>
       </c>
-      <c r="R833" t="s">
+      <c r="R834" t="s">
         <v>307</v>
       </c>
-      <c r="S833">
+      <c r="S834">
         <f>-9.2/1000</f>
         <v>-9.1999999999999998E-3</v>
       </c>
-      <c r="T833" t="s">
+      <c r="T834" t="s">
         <v>309</v>
       </c>
-      <c r="V833" t="s">
+      <c r="V834" t="s">
         <v>313</v>
-      </c>
-    </row>
-    <row r="835" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="I835" t="s">
-        <v>107</v>
-      </c>
-      <c r="R835" t="s">
-        <v>315</v>
-      </c>
-      <c r="S835" s="31">
-        <v>-0.5</v>
-      </c>
-      <c r="T835" t="s">
-        <v>310</v>
-      </c>
-      <c r="V835" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="836" spans="4:22" x14ac:dyDescent="0.25">
       <c r="I836" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R836" t="s">
         <v>315</v>
       </c>
       <c r="S836" s="31">
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="T836" t="s">
         <v>310</v>
@@ -15096,113 +15111,130 @@
     </row>
     <row r="837" spans="4:22" x14ac:dyDescent="0.25">
       <c r="I837" t="s">
-        <v>208</v>
+        <v>108</v>
       </c>
       <c r="R837" t="s">
         <v>315</v>
       </c>
-      <c r="S837" s="22">
+      <c r="S837" s="31">
         <v>-1</v>
       </c>
       <c r="T837" t="s">
         <v>310</v>
       </c>
-      <c r="U837" t="s">
+      <c r="V837" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="838" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I838" t="s">
+        <v>208</v>
+      </c>
+      <c r="R838" t="s">
+        <v>315</v>
+      </c>
+      <c r="S838" s="22">
+        <v>-1</v>
+      </c>
+      <c r="T838" t="s">
+        <v>310</v>
+      </c>
+      <c r="U838" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="838" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="R838" t="s">
+    <row r="839" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="R839" t="s">
         <v>317</v>
       </c>
-      <c r="S838" s="22">
+      <c r="S839" s="22">
         <f>-0.4 / ( (2*30.97) / (2*30.97 + 5*16) )</f>
         <v>-0.91662899580238943</v>
       </c>
-      <c r="T838" t="s">
+      <c r="T839" t="s">
         <v>318</v>
       </c>
-      <c r="U838" s="32" t="s">
+      <c r="U839" s="32" t="s">
         <v>333</v>
       </c>
-      <c r="V838" t="s">
+      <c r="V839" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="839" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="R839" t="s">
+    <row r="840" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="R840" t="s">
         <v>316</v>
       </c>
-      <c r="S839" s="22">
+      <c r="S840" s="22">
         <f>0.6 / ( (2*39.1) / (2*39.1 + 16) )</f>
         <v>0.72276214833759589</v>
       </c>
-      <c r="T839" t="s">
+      <c r="T840" t="s">
         <v>318</v>
       </c>
-      <c r="U839" s="32" t="s">
+      <c r="U840" s="32" t="s">
         <v>334</v>
       </c>
-      <c r="V839" t="s">
+      <c r="V840" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="841" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="R841" t="s">
+    <row r="842" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="R842" t="s">
         <v>308</v>
       </c>
-      <c r="S841" s="31">
+      <c r="S842" s="31">
         <f>3/5</f>
         <v>0.6</v>
       </c>
-      <c r="T841" t="s">
+      <c r="T842" t="s">
         <v>310</v>
       </c>
-      <c r="U841" t="s">
+      <c r="U842" t="s">
         <v>314</v>
       </c>
-      <c r="V841" t="s">
+      <c r="V842" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="843" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="I843" t="s">
+    <row r="844" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I844" t="s">
         <v>325</v>
       </c>
-      <c r="Q843" t="s">
+      <c r="Q844" t="s">
         <v>329</v>
       </c>
-      <c r="R843" t="s">
+      <c r="R844" t="s">
         <v>331</v>
       </c>
-      <c r="S843" s="31">
+      <c r="S844" s="31">
         <f>0.12*(44/12)</f>
         <v>0.43999999999999995</v>
       </c>
-      <c r="T843" t="s">
+      <c r="T844" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="844" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="I844" t="s">
+    <row r="845" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="I845" t="s">
         <v>339</v>
       </c>
-      <c r="Q844" t="s">
+      <c r="Q845" t="s">
         <v>329</v>
       </c>
-      <c r="R844" t="s">
+      <c r="R845" t="s">
         <v>331</v>
       </c>
-      <c r="S844" s="31">
+      <c r="S845" s="31">
         <f>0.13*(44/12)</f>
         <v>0.47666666666666668</v>
       </c>
-      <c r="T844" t="s">
+      <c r="T845" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="845" spans="4:22" x14ac:dyDescent="0.25">
-      <c r="S845" s="11"/>
+    <row r="846" spans="4:22" x14ac:dyDescent="0.25">
+      <c r="S846" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Corrected use of 'Lentils' instead of 'Lentils, dry'
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2532" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2532" uniqueCount="361">
   <si>
     <t>f_crop</t>
   </si>
@@ -820,9 +820,6 @@
   </si>
   <si>
     <t>same as pea</t>
-  </si>
-  <si>
-    <t>Lentils</t>
   </si>
   <si>
     <t>assumed to be the same as "åkerbönor"</t>
@@ -1613,13 +1610,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>174</v>
@@ -1655,7 +1652,7 @@
         <v>189</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>112</v>
@@ -1878,7 +1875,7 @@
         <v>98</v>
       </c>
       <c r="I15" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="R15" s="4" t="s">
         <v>211</v>
@@ -1890,7 +1887,7 @@
         <v>210</v>
       </c>
       <c r="U15" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
@@ -1932,7 +1929,7 @@
         <v>98</v>
       </c>
       <c r="I19" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="R19" s="4" t="s">
         <v>212</v>
@@ -1944,7 +1941,7 @@
         <v>213</v>
       </c>
       <c r="U19" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -1971,7 +1968,7 @@
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1997,7 +1994,7 @@
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="R24" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="S24">
         <v>66</v>
@@ -2006,15 +2003,15 @@
         <v>97</v>
       </c>
       <c r="U24" t="s">
+        <v>298</v>
+      </c>
+      <c r="V24" t="s">
         <v>299</v>
-      </c>
-      <c r="V24" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -2040,7 +2037,7 @@
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
@@ -2066,7 +2063,7 @@
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -2092,7 +2089,7 @@
     </row>
     <row r="29" spans="1:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
@@ -2118,7 +2115,7 @@
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -4037,7 +4034,7 @@
         <v>18.5</v>
       </c>
       <c r="U153" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="154" spans="1:22" x14ac:dyDescent="0.25">
@@ -4094,7 +4091,7 @@
         <v>12</v>
       </c>
       <c r="U155" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="156" spans="1:22" x14ac:dyDescent="0.25">
@@ -4566,7 +4563,7 @@
         <v>1.3846000000000001</v>
       </c>
       <c r="U174" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="175" spans="1:22" x14ac:dyDescent="0.25">
@@ -4805,7 +4802,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="U183" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="V183" s="8"/>
     </row>
@@ -4890,7 +4887,7 @@
         <v>3.3332999999999999</v>
       </c>
       <c r="U186" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="187" spans="1:22" x14ac:dyDescent="0.25">
@@ -4943,7 +4940,7 @@
         <v>3.3332999999999999</v>
       </c>
       <c r="U188" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="189" spans="1:22" x14ac:dyDescent="0.25">
@@ -5040,10 +5037,10 @@
         <v>65</v>
       </c>
       <c r="U192" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="V192" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="193" spans="1:22" x14ac:dyDescent="0.25">
@@ -5149,7 +5146,7 @@
         <v>4.2</v>
       </c>
       <c r="V196" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="197" spans="1:22" x14ac:dyDescent="0.25">
@@ -5176,7 +5173,7 @@
         <v>3.3</v>
       </c>
       <c r="V197" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="198" spans="1:22" x14ac:dyDescent="0.25">
@@ -5204,7 +5201,7 @@
         <v>3.75</v>
       </c>
       <c r="U198" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="199" spans="1:22" x14ac:dyDescent="0.25">
@@ -5358,7 +5355,7 @@
         <v>20</v>
       </c>
       <c r="U204" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="205" spans="1:22" x14ac:dyDescent="0.25">
@@ -5950,10 +5947,10 @@
         <v>60</v>
       </c>
       <c r="U228" t="s">
+        <v>341</v>
+      </c>
+      <c r="V228" t="s">
         <v>342</v>
-      </c>
-      <c r="V228" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="229" spans="1:22" x14ac:dyDescent="0.25">
@@ -5972,7 +5969,7 @@
         <v>30</v>
       </c>
       <c r="U229" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="230" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -5991,7 +5988,7 @@
     </row>
     <row r="231" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="4" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="R231" s="4" t="s">
         <v>243</v>
@@ -6000,7 +5997,7 @@
         <v>25</v>
       </c>
       <c r="U231" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="232" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -6014,7 +6011,7 @@
         <v>25</v>
       </c>
       <c r="U232" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="233" spans="1:22" x14ac:dyDescent="0.25">
@@ -6050,19 +6047,19 @@
     </row>
     <row r="235" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A235" s="19" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B235" s="4"/>
     </row>
     <row r="236" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A236" s="19" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B236" s="4"/>
     </row>
     <row r="237" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A237" s="19" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B237" s="4"/>
     </row>
@@ -6079,7 +6076,7 @@
         <v>245</v>
       </c>
       <c r="U238" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="V238" t="s">
         <v>250</v>
@@ -6107,7 +6104,7 @@
     </row>
     <row r="241" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B241" s="15"/>
       <c r="C241" s="15"/>
@@ -7543,7 +7540,7 @@
         <v>3</v>
       </c>
       <c r="U338" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="339" spans="1:21" x14ac:dyDescent="0.25">
@@ -7690,7 +7687,7 @@
         <v>3</v>
       </c>
       <c r="U346" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="347" spans="1:21" x14ac:dyDescent="0.25">
@@ -8154,7 +8151,7 @@
         <v>3</v>
       </c>
       <c r="U379" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="380" spans="1:21" x14ac:dyDescent="0.25">
@@ -8829,7 +8826,7 @@
         <v>20</v>
       </c>
       <c r="U430" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="431" spans="1:21" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -9022,10 +9019,10 @@
         <v>25</v>
       </c>
       <c r="U443" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="V443" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="444" spans="1:22" x14ac:dyDescent="0.25">
@@ -9382,7 +9379,7 @@
         <v>10</v>
       </c>
       <c r="V474" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="475" spans="1:22" x14ac:dyDescent="0.25">
@@ -9443,7 +9440,7 @@
         <v>15</v>
       </c>
       <c r="V479" s="25" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="480" spans="1:22" x14ac:dyDescent="0.25">
@@ -9461,7 +9458,7 @@
         <v>15</v>
       </c>
       <c r="U480" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="481" spans="1:22" x14ac:dyDescent="0.25">
@@ -9479,7 +9476,7 @@
         <v>15</v>
       </c>
       <c r="U481" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="482" spans="1:22" x14ac:dyDescent="0.25">
@@ -9502,7 +9499,7 @@
         <v>0.6</v>
       </c>
       <c r="V483" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="484" spans="1:22" x14ac:dyDescent="0.25">
@@ -9519,7 +9516,7 @@
         <v>1.6</v>
       </c>
       <c r="V484" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="485" spans="1:22" x14ac:dyDescent="0.25">
@@ -9537,7 +9534,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="U485" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="486" spans="1:22" x14ac:dyDescent="0.25">
@@ -9788,7 +9785,7 @@
     </row>
     <row r="501" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A501" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B501" s="15"/>
       <c r="C501" s="15"/>
@@ -9814,7 +9811,7 @@
     </row>
     <row r="502" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A502" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B502" s="2"/>
       <c r="C502" s="2"/>
@@ -9840,7 +9837,7 @@
     </row>
     <row r="503" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A503" s="19" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B503" s="19"/>
       <c r="C503" s="19"/>
@@ -9848,7 +9845,7 @@
     </row>
     <row r="504" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A504" s="19" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B504" s="19"/>
       <c r="C504" s="19"/>
@@ -10904,7 +10901,7 @@
         <v>5</v>
       </c>
       <c r="U577" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="578" spans="1:21" x14ac:dyDescent="0.25">
@@ -11015,7 +11012,7 @@
         <v>5</v>
       </c>
       <c r="U583" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="584" spans="1:21" x14ac:dyDescent="0.25">
@@ -11365,7 +11362,7 @@
         <v>37</v>
       </c>
       <c r="P609" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R609" t="s">
         <v>205</v>
@@ -11421,7 +11418,7 @@
         <v>37</v>
       </c>
       <c r="P613" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R613" t="s">
         <v>206</v>
@@ -11445,7 +11442,7 @@
         <v>10</v>
       </c>
       <c r="U614" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="615" spans="1:21" x14ac:dyDescent="0.25">
@@ -11483,7 +11480,7 @@
         <v>67</v>
       </c>
       <c r="P617" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R617" t="s">
         <v>205</v>
@@ -11543,7 +11540,7 @@
         <v>67</v>
       </c>
       <c r="P621" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R621" t="s">
         <v>206</v>
@@ -11608,7 +11605,7 @@
         <v>39</v>
       </c>
       <c r="P627" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R627" t="s">
         <v>205</v>
@@ -11664,7 +11661,7 @@
         <v>39</v>
       </c>
       <c r="P631" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R631" t="s">
         <v>206</v>
@@ -11728,7 +11725,7 @@
         <v>33</v>
       </c>
       <c r="P637" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R637" t="s">
         <v>205</v>
@@ -11784,7 +11781,7 @@
         <v>33</v>
       </c>
       <c r="P641" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R641" t="s">
         <v>206</v>
@@ -11843,7 +11840,7 @@
         <v>34</v>
       </c>
       <c r="P645" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R645" t="s">
         <v>205</v>
@@ -11903,7 +11900,7 @@
         <v>34</v>
       </c>
       <c r="P649" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R649" t="s">
         <v>206</v>
@@ -11915,7 +11912,7 @@
     </row>
     <row r="651" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A651" s="21" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B651" s="21"/>
       <c r="C651" s="21"/>
@@ -11978,7 +11975,7 @@
         <v>50</v>
       </c>
       <c r="U655" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="656" spans="1:21" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12103,7 +12100,7 @@
         <v>35</v>
       </c>
       <c r="P664" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R664" t="s">
         <v>206</v>
@@ -12157,10 +12154,10 @@
         <v>155</v>
       </c>
       <c r="U667" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="V667" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="668" spans="1:22" x14ac:dyDescent="0.25">
@@ -12513,7 +12510,7 @@
         <v>20</v>
       </c>
       <c r="V698" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="699" spans="1:22" x14ac:dyDescent="0.25">
@@ -12574,7 +12571,7 @@
         <v>105</v>
       </c>
       <c r="V703" s="25" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="704" spans="1:22" x14ac:dyDescent="0.25">
@@ -12592,7 +12589,7 @@
         <v>105</v>
       </c>
       <c r="U704" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="705" spans="1:22" x14ac:dyDescent="0.25">
@@ -12610,7 +12607,7 @@
         <v>105</v>
       </c>
       <c r="U705" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="706" spans="1:22" x14ac:dyDescent="0.25">
@@ -12633,7 +12630,7 @@
         <v>5.6</v>
       </c>
       <c r="V707" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="708" spans="1:22" x14ac:dyDescent="0.25">
@@ -12650,7 +12647,7 @@
         <v>3</v>
       </c>
       <c r="V708" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="709" spans="1:22" x14ac:dyDescent="0.25">
@@ -12668,7 +12665,7 @@
         <v>4.3</v>
       </c>
       <c r="U709" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="710" spans="1:22" x14ac:dyDescent="0.25">
@@ -12739,7 +12736,7 @@
     </row>
     <row r="715" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A715" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B715" s="2"/>
       <c r="C715" s="2"/>
@@ -12772,7 +12769,7 @@
       </c>
       <c r="T717" s="5"/>
       <c r="U717" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="719" spans="1:22" x14ac:dyDescent="0.25">
@@ -12820,7 +12817,7 @@
     </row>
     <row r="721" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A721" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B721" s="1"/>
       <c r="C721" s="1"/>
@@ -14527,7 +14524,7 @@
         <v>148</v>
       </c>
       <c r="R797" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="S797" s="35">
         <f>S796</f>
@@ -14537,12 +14534,12 @@
         <v>109</v>
       </c>
       <c r="U797" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="799" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A799" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B799" s="2"/>
       <c r="C799" s="2"/>
@@ -14574,7 +14571,7 @@
         <v>0</v>
       </c>
       <c r="T800" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="U800" s="5" t="s">
         <v>12</v>
@@ -14605,7 +14602,7 @@
         <v>175</v>
       </c>
       <c r="Q803" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="R803" t="s">
         <v>166</v>
@@ -14615,10 +14612,10 @@
         <v>22366.666666666664</v>
       </c>
       <c r="T803" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V803" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="804" spans="1:22" x14ac:dyDescent="0.25">
@@ -14626,7 +14623,7 @@
         <v>175</v>
       </c>
       <c r="Q804" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="R804" t="s">
         <v>166</v>
@@ -14636,10 +14633,10 @@
         <v>58.3</v>
       </c>
       <c r="T804" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="V804" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="806" spans="1:22" x14ac:dyDescent="0.25">
@@ -14659,10 +14656,10 @@
         <v>167</v>
       </c>
       <c r="U806" t="s">
+        <v>354</v>
+      </c>
+      <c r="V806" t="s">
         <v>355</v>
-      </c>
-      <c r="V806" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="807" spans="1:22" x14ac:dyDescent="0.25">
@@ -14670,7 +14667,7 @@
         <v>176</v>
       </c>
       <c r="Q807" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="R807" t="s">
         <v>166</v>
@@ -14680,10 +14677,10 @@
         <v>9533.3333333333339</v>
       </c>
       <c r="T807" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V807" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="808" spans="1:22" x14ac:dyDescent="0.25">
@@ -14691,7 +14688,7 @@
         <v>176</v>
       </c>
       <c r="Q808" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="R808" t="s">
         <v>166</v>
@@ -14701,10 +14698,10 @@
         <v>7.9</v>
       </c>
       <c r="T808" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="V808" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="810" spans="1:22" x14ac:dyDescent="0.25">
@@ -14795,7 +14792,7 @@
     </row>
     <row r="816" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A816" s="27" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B816" s="27"/>
       <c r="C816" s="28"/>
@@ -14821,10 +14818,10 @@
     </row>
     <row r="818" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I818" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R818" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="S818" s="11">
         <f>213/(213 + 60)*100</f>
@@ -14834,15 +14831,15 @@
         <v>97</v>
       </c>
       <c r="V818" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="819" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I819" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="R819" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="S819" s="11">
         <f>60/(213 + 60)*100</f>
@@ -14852,15 +14849,15 @@
         <v>97</v>
       </c>
       <c r="V819" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="821" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I821" t="s">
+        <v>324</v>
+      </c>
+      <c r="R821" t="s">
         <v>325</v>
-      </c>
-      <c r="R821" t="s">
-        <v>326</v>
       </c>
       <c r="S821">
         <v>45</v>
@@ -14869,15 +14866,15 @@
         <v>97</v>
       </c>
       <c r="V821" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="822" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I822" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="R822" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="S822">
         <v>48</v>
@@ -14886,25 +14883,25 @@
         <v>97</v>
       </c>
       <c r="V822" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="824" spans="1:22" x14ac:dyDescent="0.25">
       <c r="R824" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S824" s="30">
         <f>S831</f>
         <v>-5.9999999999999995E-4</v>
       </c>
       <c r="T824" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U824" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="V824" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="825" spans="1:22" x14ac:dyDescent="0.25">
@@ -14915,20 +14912,20 @@
         <v>142</v>
       </c>
       <c r="R825" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S825" s="29">
         <f>-(45.5*0.1+10.7*0.9)/1000</f>
         <v>-1.418E-2</v>
       </c>
       <c r="T825" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U825" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="V825" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="826" spans="1:22" x14ac:dyDescent="0.25">
@@ -14939,14 +14936,14 @@
         <v>142</v>
       </c>
       <c r="R826" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S826" s="33">
         <f>S825</f>
         <v>-1.418E-2</v>
       </c>
       <c r="T826" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="827" spans="1:22" x14ac:dyDescent="0.25">
@@ -14957,20 +14954,20 @@
         <v>98</v>
       </c>
       <c r="R827" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S827" s="29">
         <f>-(45.5*0.4+10.7*0.6)/1000</f>
         <v>-2.4619999999999996E-2</v>
       </c>
       <c r="T827" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U827" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="V827" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="828" spans="1:22" x14ac:dyDescent="0.25">
@@ -14981,14 +14978,14 @@
         <v>98</v>
       </c>
       <c r="R828" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S828" s="33">
         <f>S827</f>
         <v>-2.4619999999999996E-2</v>
       </c>
       <c r="T828" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="829" spans="1:22" x14ac:dyDescent="0.25">
@@ -14997,20 +14994,20 @@
       </c>
       <c r="B829" s="4"/>
       <c r="R829" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S829" s="4">
         <f>-10.7/1000</f>
         <v>-1.0699999999999999E-2</v>
       </c>
       <c r="T829" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U829" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="V829" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="830" spans="1:22" x14ac:dyDescent="0.25">
@@ -15019,20 +15016,20 @@
       </c>
       <c r="B830" s="4"/>
       <c r="R830" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S830" s="4">
         <f>-10.7/1000</f>
         <v>-1.0699999999999999E-2</v>
       </c>
       <c r="T830" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U830" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="V830" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="831" spans="1:22" x14ac:dyDescent="0.25">
@@ -15040,56 +15037,56 @@
         <v>226</v>
       </c>
       <c r="R831" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S831">
         <f>-0.6/1000</f>
         <v>-5.9999999999999995E-4</v>
       </c>
       <c r="T831" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="V831" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="832" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B832" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="R832" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="S832" s="29">
         <f>-20*0.45/0.85/1000</f>
         <v>-1.0588235294117647E-2</v>
       </c>
       <c r="T832" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="U832" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="V832" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="834" spans="4:22" x14ac:dyDescent="0.25">
       <c r="D834" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="R834" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="S834">
         <f>-9.2/1000</f>
         <v>-9.1999999999999998E-3</v>
       </c>
       <c r="T834" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="V834" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="836" spans="4:22" x14ac:dyDescent="0.25">
@@ -15097,16 +15094,16 @@
         <v>107</v>
       </c>
       <c r="R836" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="S836" s="31">
         <v>-0.5</v>
       </c>
       <c r="T836" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="V836" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="837" spans="4:22" x14ac:dyDescent="0.25">
@@ -15114,16 +15111,16 @@
         <v>108</v>
       </c>
       <c r="R837" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="S837" s="31">
         <v>-1</v>
       </c>
       <c r="T837" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="V837" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="838" spans="4:22" x14ac:dyDescent="0.25">
@@ -15131,106 +15128,106 @@
         <v>208</v>
       </c>
       <c r="R838" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="S838" s="22">
         <v>-1</v>
       </c>
       <c r="T838" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="U838" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="839" spans="4:22" x14ac:dyDescent="0.25">
       <c r="R839" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="S839" s="22">
         <f>-0.4 / ( (2*30.97) / (2*30.97 + 5*16) )</f>
         <v>-0.91662899580238943</v>
       </c>
       <c r="T839" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="U839" s="32" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="V839" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="840" spans="4:22" x14ac:dyDescent="0.25">
       <c r="R840" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="S840" s="22">
         <f>0.6 / ( (2*39.1) / (2*39.1 + 16) )</f>
         <v>0.72276214833759589</v>
       </c>
       <c r="T840" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="U840" s="32" t="s">
+        <v>333</v>
+      </c>
+      <c r="V840" t="s">
         <v>334</v>
-      </c>
-      <c r="V840" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="842" spans="4:22" x14ac:dyDescent="0.25">
       <c r="R842" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="S842" s="31">
         <f>3/5</f>
         <v>0.6</v>
       </c>
       <c r="T842" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="U842" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="V842" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="844" spans="4:22" x14ac:dyDescent="0.25">
       <c r="I844" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="Q844" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="R844" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="S844" s="31">
         <f>0.12*(44/12)</f>
         <v>0.43999999999999995</v>
       </c>
       <c r="T844" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="845" spans="4:22" x14ac:dyDescent="0.25">
       <c r="I845" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="Q845" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="R845" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="S845" s="31">
         <f>0.13*(44/12)</f>
         <v>0.47666666666666668</v>
       </c>
       <c r="T845" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="846" spans="4:22" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added liming effect of non-manure organic fertilisers through parameter 'lime_effect_organic' in PlandNutrientMgmt
</commit_message>
<xml_diff>
--- a/data/default/PlantNutrientMgmt.xlsx
+++ b/data/default/PlantNutrientMgmt.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D849481-FAFA-4D35-9359-07E2CC878DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3657ADE9-7677-4025-8F26-7588A230C27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35805" yWindow="2595" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1755" yWindow="870" windowWidth="21600" windowHeight="13785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2505" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2508" uniqueCount="363">
   <si>
     <t>f_crop</t>
   </si>
@@ -1111,6 +1111,15 @@
   </si>
   <si>
     <t>Use factor from Finland. Sweden uses a more sophisticated model for N leaching</t>
+  </si>
+  <si>
+    <t>lime_effect_organic</t>
+  </si>
+  <si>
+    <t>kg CaO/kg P</t>
+  </si>
+  <si>
+    <t>Lime effect of non-manure organic fertiliser assumed same as manure</t>
   </si>
 </sst>
 </file>
@@ -1582,7 +1591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V842"/>
+  <dimension ref="A1:V843"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="21" customWidth="1"/>
@@ -15035,7 +15044,7 @@
         <v>-0.91662899580238943</v>
       </c>
       <c r="T835" t="s">
-        <v>312</v>
+        <v>361</v>
       </c>
       <c r="U835" s="27" t="s">
         <v>327</v>
@@ -15080,44 +15089,59 @@
         <v>307</v>
       </c>
     </row>
-    <row r="840" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="I840" t="s">
+    <row r="839" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="R839" t="s">
+        <v>360</v>
+      </c>
+      <c r="S839" s="26">
+        <f>3/5</f>
+        <v>0.6</v>
+      </c>
+      <c r="T839" t="s">
+        <v>304</v>
+      </c>
+      <c r="U839" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="841" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="I841" t="s">
         <v>319</v>
       </c>
-      <c r="Q840" t="s">
+      <c r="Q841" t="s">
         <v>323</v>
       </c>
-      <c r="R840" t="s">
+      <c r="R841" t="s">
         <v>325</v>
       </c>
-      <c r="S840" s="26">
+      <c r="S841" s="26">
         <f>0.12*(44/12)</f>
         <v>0.43999999999999995</v>
       </c>
-      <c r="T840" t="s">
+      <c r="T841" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="841" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="I841" t="s">
+    <row r="842" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="I842" t="s">
         <v>333</v>
       </c>
-      <c r="Q841" t="s">
+      <c r="Q842" t="s">
         <v>323</v>
       </c>
-      <c r="R841" t="s">
+      <c r="R842" t="s">
         <v>325</v>
       </c>
-      <c r="S841" s="26">
+      <c r="S842" s="26">
         <f>0.13*(44/12)</f>
         <v>0.47666666666666668</v>
       </c>
-      <c r="T841" t="s">
+      <c r="T842" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="842" spans="9:22" x14ac:dyDescent="0.25">
-      <c r="S842" s="9"/>
+    <row r="843" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="S843" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>